<commit_message>
Fix scripts and ignore output files
</commit_message>
<xml_diff>
--- a/src/results/(News)Sentiment.xlsx
+++ b/src/results/(News)Sentiment.xlsx
@@ -3,12 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="3" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)All" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Bioenergi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Energi Fosil" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Harga Minyak" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Volume Minyak" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Harga Produk Kilang" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Volume Produk Kilang" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -17,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -121,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -130,18 +132,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1151,31 +1149,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Tanggal awal</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Tanggal akhir</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="n">
+      <c r="A2" s="7" t="n">
         <v>45950</v>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="7" t="n">
         <v>45957</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1185,10 +1183,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n">
+      <c r="A3" s="7" t="n">
         <v>45958</v>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="7" t="n">
         <v>45973</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1201,17 +1199,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
-        <v>45973</v>
-      </c>
-      <c r="B4" s="9" t="n">
-        <v>45987</v>
+      <c r="A4" s="7" t="n">
+        <v>45974</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>45981</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1. Harga minyak kelapa sawit (CPO) mengalami penurunan signifikan antara tanggal 21 hingga 24 November 2025, mencapai level terendah dalam lebih dari empat bulan, disebabkan oleh peningkatan pasokan di Malaysia, perkiraan lesunya permintaan ekspor, apresiasi nilai tukar ringgit, dan penurunan harga minyak nabati pesaing.
-2. Meskipun berada dalam zona bearish, analisis teknikal harian dan mingguan menunjukkan potensi CPO untuk mengalami technical rebound atau kenaikan harga dalam waktu dekat, mengingat komoditas tersebut telah terkoreksi dalam dan berada dalam kondisi jenuh jual (oversold).
-3. Kementerian Kehutanan (Kemenhut) dan Satuan Tugas Penertiban Kawasan Hutan (Satgas PKH) memperketat pengamanan dan melanjutkan operasi penertiban kebun sawit ilegal di Taman Nasional Tesso Nilo, Riau, dengan fokus mengembalikan kawasan sebagai habitat gajah sumatera dan menindak pemilik lahan, pemodal, serta pengendali alat berat, bukan masyarakat kecil, meskipun menghadapi perusakan fasilitas posko.</t>
+          <t>1. Beberapa perusahaan kelapa sawit menunjukkan kinerja keuangan yang membaik, di mana PTPN IV PalmCo melaporkan peningkatan laba bersih 49% menjadi Rp3,76 triliun pada tahun 2024, dan PT Sampoerna Agro Tbk (SGRO) mengalami kenaikan laba bersih 236,06% pada semester I-2025 yang diikuti akuisisi oleh POSCO International. Selain itu, PT Sawit Sumbermas Sarana Tbk (SSMS) memperoleh pembiayaan sindikasi Rp5,2 triliun untuk memperkuat operasional dan ekspansi melalui akuisisi lahan.
+2. Harga minyak sawit mentah (CPO) di Bursa Malaysia sempat naik selama lima hari berturut-turut hingga mencapai MYR 4.226/ton pada 19 November 2025, namun kemudian reli tersebut terhenti akibat permintaan yang melemah dan penurunan harga minyak kedelai. Sejalan dengan perbaikan harga CPO, harga tandan buah segar (TBS) sawit petani mitra di Sumatra Utara sedikit meningkat menjadi Rp3.435,79 per kilogram, meskipun harga kernel mengalami penurunan.
+3. Sektor kelapa sawit Indonesia terus berupaya memenuhi standar keberlanjutan global, ditunjukkan dengan peluncuran ESG Advisory Playbook oleh BNI untuk membantu debitur dalam transisi hijau. Di sisi lain, meskipun Indonesia–European Union Comprehensive Economic Partnership Agreement (IEU-CEPA) diharapkan menghapus tarif ekspor, produk sawit masih menghadapi tantangan ketat dari regulasi keberlanjutan Uni Eropa seperti EUDR dan RED, yang memerlukan perbaikan rantai pasok dan ketelusuran untuk mempertahankan akses pasar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>45986</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1. Harga minyak sawit mentah (CPO) menunjukkan tren penurunan pada periode ini, dengan harga di Bursa Malaysia Derivatives Exchange tercatat turun menjadi MYR 4.068/ton pada 21 November dan MYR 4.055/ton pada 24 November. Penurunan harga ini disebabkan oleh beberapa faktor, termasuk peningkatan inventori pasokan, perkiraan permintaan ekspor yang melemah dari Malaysia, penguatan nilai tukar ringgit yang membuat CPO lebih mahal bagi pembeli asing, serta harga minyak nabati pesaing seperti minyak kedelai yang juga mengalami penurunan.
+2. Indonesia diproyeksikan akan mengalami penurunan porsi ekspor sawitnya di masa mendatang karena peningkatan utilisasi domestik. Kebutuhan dalam negeri akan sawit semakin besar, terutama untuk mendukung program mandatory biodiesel B40. Ekonom menyarankan agar pemerintah melakukan perhitungan yang tepat untuk memastikan pasokan CPO dapat memenuhi kebutuhan B40 tanpa mengorbankan pasokan untuk industri dan rumah tangga. Ada juga peluang untuk meningkatkan produktivitas CPO melalui peremajaan sawit tanpa perlu menambah luas lahan, dengan memanfaatkan dana Badan Pengelola Dana Perkebunan Kelapa Sawit (BPDPKS).
+3. Sektor hilirisasi sawit nasional mengalami perkembangan dengan diresmikannya PT AGPA Refinery Complex (ARC) di Balikpapan, Kalimantan Timur. Fasilitas dengan kapasitas 500.000 ton per tahun ini merupakan hasil kolaborasi Indonesia-Korea Selatan dan bertujuan untuk memperkuat rantai pasok energi bersih berbasis kelapa sawit. ARC diharapkan dapat menciptakan nilai tambah bagi industri sawit nasional dengan mengolah CPO menjadi berbagai produk bernilai jual tinggi seperti minyak nabati dan bahan bakar bio, yang sebagian besar ditujukan untuk ekspor, serta mendukung transisi menuju energi bersih.</t>
         </is>
       </c>
     </row>
@@ -1226,31 +1239,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Tanggal awal</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Tanggal akhir</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="n">
+      <c r="A2" s="7" t="n">
         <v>45967</v>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="7" t="n">
         <v>45974</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1260,10 +1273,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n">
+      <c r="A3" s="7" t="n">
         <v>45975</v>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="7" t="n">
         <v>45980</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1276,18 +1289,292 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="7" t="n">
+        <v>45981</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>45981</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1.  Persediaan produk olahan seperti bensin dan distilat (termasuk solar) di Amerika Serikat, setelah periode di level rendah dalam lebih dari satu dekade, baru-baru ini mencatat kenaikan untuk pertama kalinya dalam lebih dari sebulan. Meskipun demikian, selisih harga produk olahan (crack spreads) tetap tinggi. Sementara itu, harga gas alam di AS mengalami kenaikan hampir dua kali lipat tahun ini karena permintaan yang tinggi, sedangkan harga gas alam di Eropa cenderung rendah.
+2.  Harga minyak mentah global menunjukkan tren melemah, dengan Brent diperdagangkan di bawah $64 per barel dan WTI di atas $59 per barel, didominasi sentimen pasokan yang cenderung surplus. Meskipun persediaan minyak mentah AS menurun, volume minyak yang diangkut melalui laut meningkat tajam, mencapai rekor tertinggi, sebagian karena rute transit yang lebih panjang untuk minyak Rusia.
+3.  Di Indonesia, Pertamina memperkuat pengawasan pasokan BBM dan LPG untuk menghadapi lonjakan permintaan dan tantangan cuaca ekstrem menjelang periode libur akhir tahun 2025 dan awal 2026. Proyek Refinery Development Master Plan (RDMP) Balikpapan dijadwalkan akan diresmikan pada pertengahan Desember 2025, yang diharapkan mengurangi ketergantungan impor BBM hingga 15% dengan kapasitas produksi 360.000 barel per hari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>45986</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1. Harga minyak global menunjukkan tren penurunan dengan Brent Crude dan WTI masing-masing berada di sekitar $62.59 dan $58.08 per barel, dipicu laporan kesepakatan damai Ukraina-AS dan kekhawatiran pasokan berlebih. Harga gas Eropa juga turun ke level terendah sejak Mei 2024 karena negosiasi damai, cuaca hangat, dan pasokan yang melimpah. Analis memproyeksikan penurunan harga lebih lanjut hingga 2026-2027, meskipun ada kekhawatiran tentang kurangnya investasi dalam jangka panjang.
+2. Pasokan bahan bakar minyak (BBM) di SPBU swasta di Indonesia, seperti Vivo, BP-AKR, dan Shell, berangsur pulih setelah melakukan pembelian base fuel dari Pertamina Patra Niaga. Vivo telah membeli 100.000 barel dan menurunkan harga Revvo 92, sementara BP-AKR menambah pasokan menjadi total 200.000 barel, dan Shell telah menyelesaikan negosiasi untuk pembelian 100.000 barel.
+3. Pemerintah Indonesia melakukan langkah-langkah untuk mendukung Pertamina dan ketahanan energi nasional, termasuk mengubah skema pencairan dana kompensasi BBM bersubsidi menjadi bulanan yang akan mendukung likuiditas Pertamina. Pertamina Patra Niaga juga meningkatkan stok Pertalite sebesar 1,4 juta kiloliter dan menyiapkan satuan tugas untuk memastikan ketersediaan BBM selama periode Natal dan Tahun Baru (Nataru), serta berupaya menjaga keterjangkauan harga BBM campuran bioetanol melalui relaksasi cukai.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal awal</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal akhir</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>45967</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>45974</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B3" s="7" t="n">
         <v>45980</v>
       </c>
-      <c r="B4" s="9" t="n">
-        <v>45987</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1.  Pasar minyak global saat ini ditandai oleh kelebihan pasokan yang signifikan, dengan IEA dan OPEC memproyeksikan surplus besar pada tahun 2026, diperparah oleh peningkatan stok minyak mentah AS, yang menyebabkan harga minyak bertahan di level rendah meskipun ada gangguan geopolitik jangka pendek.
+2.  Ketegangan geopolitik, khususnya perang Rusia-Ukraina, terus memengaruhi pasokan minyak global, di mana serangan drone Ukraina di pelabuhan dan kilang minyak Rusia menyebabkan gangguan ekspor sementara, sementara sanksi AS yang akan datang terhadap produsen Rusia memperlebar diskon minyak mentah Urals secara signifikan terhadap Brent.
+3.  Di Indonesia, sektor energi fosil menghadapi isu hukum terkait dugaan korupsi impor BBM yang melibatkan mantan pejabat Pertamina Patra Niaga, di mana tim kuasa hukum berargumen bahwa kliennya justru mencetak keuntungan historis bagi perusahaan.
+4.  Pemerintah Indonesia melalui Kementerian ESDM juga mendorong penerapan bensin campuran etanol 10% (E10) pada tahun 2028 meskipun menghadapi berbagai tantangan, sementara Pertamina Patra Niaga berhasil mengendalikan penyaluran BBM bersubsidi dengan memblokir ratusan ribu kendaraan yang terindikasi melakukan kecurangan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>45981</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>45981</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1. Pasokan bahan bakar minyak (BBM) di SPBU swasta seperti Shell, BP-AKR, dan Vivo diperkirakan akan kembali normal pada akhir November 2025. Hal ini menyusul kesepakatan pembelian *base fuel* (bahan bakar murni) dari PT Pertamina Patra Niaga, dengan Shell dan Vivo masing-masing menyerap 100.000 barel, sementara BP-AKR menambah pasokan hingga total 200.000 barel.
-2. PT Pertamina Patra Niaga meningkatkan stok BBM nasional, termasuk Pertalite sebanyak 1,4 juta kiloliter dan Pertamax Turbo, untuk mengamankan pasokan selama periode Natal dan Tahun Baru (Nataru) 2025/2026. Kementerian Pertahanan juga akan mengerahkan personel TNI mulai Desember 2025 untuk mengamankan kilang minyak dan terminal Pertamina yang merupakan objek vital nasional.
-3. Kementerian Energi dan Sumber Daya Mineral (ESDM) akan memperketat pengawasan kualitas BBM Pertamina, terutama menjelang Nataru, setelah adanya beberapa keluhan masyarakat terkait kualitas BBM yang tercampur air atau isu lainnya. Pengawasan ini akan melibatkan analisis rutin oleh Lemigas.
-4. Di pasar global, harga minyak mentah mengalami penurunan (Brent di $62/barel, WTI di $58.08/barel) karena laporan kemajuan kesepakatan damai Rusia-Ukraina dan kekhawatiran pasokan berlebih. Sementara itu, harga gas di Eropa berada pada level terendah sejak Mei 2024 akibat perundingan damai, cuaca hangat, dan pasokan yang melimpah.</t>
+          <t>1. Menjelang libur Natal 2025 dan Tahun Baru 2026, Pertamina meningkatkan pengawasan pasokan dan distribusi BBM dan LPG untuk mengantisipasi lonjakan permintaan serta potensi gangguan cuaca ekstrem. Proyek Refinery Development Master Plan (RDMP) Balikpapan, yang direncanakan beroperasi penuh pada pertengahan Desember 2025, ditargetkan mampu memangkas ketergantungan impor BBM hingga 15% dengan kapasitas produksi mencapai 360.000 barel per hari, didukung oleh fasilitas penyimpanan minyak berkapasitas 2 juta kiloliter.
+2. Ketersediaan stok BBM nasional berada dalam kondisi aman dengan cadangan dilaporkan cukup untuk 18 hingga 19 hari.
+3. Di pasar global, harga minyak mentah mempertahankan penurunan setelah persediaan bahan bakar di Amerika Serikat meningkat, meskipun data menunjukkan persediaan minyak mentah AS turun sebesar 3,4 juta barel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>45986</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.  Beberapa operator SPBU swasta, yaitu BP-AKR dan Vivo, telah memperoleh tambahan pasokan base fuel dari Pertamina Patra Niaga masing-masing 100.000 barel, sehingga total pembelian BP-AKR mencapai 200.000 barel. Shell Indonesia juga dalam tahap final negosiasi untuk membeli 100.000 barel base fuel dari Pertamina Patra Niaga untuk mengisi kembali stok BBM mereka.
+2.  Pertamina Patra Niaga meningkatkan stok Pertalite sebesar 1,4 juta kiloliter (KL) melalui kombinasi produksi kilang dan impor, dengan tujuan memperkuat ketahanan stok BBM menjadi 21-23 hari menjelang periode Natal dan Tahun Baru. Penambahan stok juga dilakukan untuk Pertamax Turbo.
+3.  Dalam upaya efisiensi dan regulasi, Daihatsu meluncurkan Rocky e-Smart Hybrid yang diklaim sangat efisien dengan konsumsi BBM 34,8 km per liter. Di sisi kebijakan, BPH Migas akan menyelesaikan revisi Perpres No. 191 Tahun 2014 untuk tata kelola penyaluran Pertalite agar lebih tepat sasaran, sementara usulan penghapusan cukai bioetanol sebesar Rp20.000 per liter juga diajukan karena saat ini menambah harga Pertamax Green 95 sekitar Rp1.000 per liter.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal awal</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal akhir</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>45950</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>45957</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>45958</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>45973</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>45974</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>45981</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1. Kilang Pertamina Internasional (KPI) telah meningkatkan kapasitas produksi unit platformer di Kilang Dumai menjadi 14 ribu barel per hari, yang menghasilkan gasoline RON 95.
+2. KPI memproduksi biofuel melalui metode co-processing, menghasilkan bioavtur Pertamina Sustainable Aviation Fuel (SAF) dengan bahan baku minyak inti sawit, serta memproduksi biodiesel 100% (HVO) atau Pertamina Renewable Diesel dari bahan baku nabati.
+3. Pengembangan green refinery oleh KPI mencakup produksi Pertamina SAF dari minyak jelantah di Kilang Cilacap, yang telah digunakan dalam penerbangan komersial perdana pada pertengahan Agustus 2025, dan berencana dikembangkan lebih lanjut di Kilang Dumai dan Balongan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>45986</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.  Menteri Pertahanan menginstruksikan pengerahan personel Tentara Nasional Indonesia (TNI) untuk mengamankan kilang minyak dan terminal milik PT Pertamina (Persero).
+2.  Pengerahan pasukan akan dimulai pada Desember 2025, dengan menugaskan personel dari TNI Angkatan Darat dan dipantau oleh Badan Intelijen Strategis (BAIS).
+3.  Kementerian Energi dan Sumber Daya Mineral (ESDM) menyatakan dukungan terhadap rencana ini, menganggapnya sebagai langkah wajar karena kilang Pertamina termasuk dalam kategori objek vital nasional.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal awal</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal akhir</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>45950</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>45957</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>45958</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>45973</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>45974</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>45981</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tidak ada berita</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>45986</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tidak ada berita</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: scrape and sentiment RUPL
</commit_message>
<xml_diff>
--- a/src/results/(News)Sentiment.xlsx
+++ b/src/results/(News)Sentiment.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="13" activeTab="14" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11280" tabRatio="600" firstSheet="13" activeTab="15" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)All" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,10 +21,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)PDB" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Biodiesel" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Bioetanol" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Harga Minyak" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Volume Minyak" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Harga Produk Kilang" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Volume Produk Kilang" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)RUPTL" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Harga Minyak" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Volume Minyak" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Harga Produk Kilang" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="(Summary)Volume Produk Kilang" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -38,13 +39,18 @@
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -73,12 +79,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -136,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -149,6 +170,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -519,7 +543,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -1163,7 +1187,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -1247,7 +1271,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -1331,7 +1355,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -1415,7 +1439,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -1499,7 +1523,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
@@ -1652,7 +1676,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="13.36328125" customWidth="1" min="1" max="1"/>
+    <col width="14.36328125" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
@@ -1677,10 +1705,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="n">
+      <c r="A2" s="1" t="n">
         <v>45990</v>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="1" t="n">
         <v>45991</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1695,10 +1723,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="1" t="n">
         <v>45998</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1715,10 +1743,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="1" t="n">
         <v>45999</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="1" t="n">
         <v>46005</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1745,151 +1773,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Tanggal awal</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Tanggal akhir</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Summary Data</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>45961</v>
+      <c r="A2" s="8" t="n">
+        <v>45990</v>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>45991</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45962</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>45968</v>
+      <c r="A3" s="8" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>45998</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1. Harga minyak mentah global mengalami tekanan penurunan sepanjang minggu pertama November 2025 akibat kekhawatiran kelebihan pasokan dan lemahnya permintaan, khususnya dari Amerika Serikat. Harga Brent diperdagangkan di sekitar US$63-US$64 per barel, dan West Texas Intermediate (WTI) mendekati US$60 per barel, dengan WTI anjlok sekitar 16-17% secara tahun berjalan. Stok minyak mentah AS menunjukkan kenaikan signifikan, dengan laporan API sebesar 6.5 juta barel dan EIA sebesar 5.2 juta barel pada pekan lalu.
-2. OPEC+ memutuskan untuk menghentikan sementara rencana kenaikan produksi pada kuartal I 2026, setelah peningkatan moderat pada Desember, sebagai upaya menyeimbangkan pasar dan meredam volatilitas. Morgan Stanley menaikkan proyeksi harga Brent menjadi US$60 per barel untuk semester I 2026 dari US$57.50. Namun, proyeksi tekanan harga tetap ada, dengan Capital Economics memperkirakan Brent mencapai US$60 per barel pada akhir 2025 dan US$50 per barel pada akhir 2026.
-3. Sanksi AS terhadap produsen minyak utama Rusia (Rosneft PJSC dan Lukoil PJSC) mengakibatkan kilang-kilang di China menghentikan pembelian minyak mentah Rusia, mempengaruhi sekitar 400.000 barel per hari atau 45% dari total impor Rusia ke China. Kondisi pasar yang cukup pasokan ini mendorong Arab Saudi untuk memangkas harga jual minyak mentah utamanya untuk pembeli Asia pada Desember, termasuk Arab Light yang dipangkas US$1.20 per barel.</t>
-        </is>
-      </c>
+          <t>1. Pemerintah dan PT PLN (Persero) mempercepat pemulihan infrastruktur kelistrikan di wilayah Sumatra (Aceh, Sumatra Utara, dan Sumatra Barat) yang terdampak bencana banjir dan longsor, dengan target sebagian besar wilayah pulih pada 6-7 Desember 2025. Proses pemulihan melibatkan pengerahan personel, pengiriman material melalui berbagai moda transportasi termasuk udara, serta dukungan dari berbagai instansi. Relaksasi aturan pembelian BBM juga diberlakukan di daerah terdampak untuk menjamin pasokan.
+2. Diskusi dan kebijakan terkait transisi energi terus berjalan, meliputi pembatalan pensiun dini PLTU Cirebon-1 dengan alasan teknis dan pencarian PLTU alternatif yang lebih tua dan berdampak lingkungan lebih buruk. Sektor panas bumi aktif dengan rencana pembentukan usaha patungan antara PT Pertamina Geothermal Energy Tbk (PGEO) dan PT PLN Indonesia Power (PLN IP) untuk menggarap proyek berkapasitas besar. Sementara itu, pengembangan energi nuklir menjadi perhatian, dengan PLN menugaskan kajian teknologi PLTN dan rencana pembentukan Badan Pelaksana Program Energi Nuklir (NEPIO) yang ditargetkan beroperasi pada 2030.
+3. Kinerja sektor batubara menunjukkan penurunan ekspor dan harga yang cenderung melemah. Pemerintah tengah mempertimbangkan penerapan bea keluar batubara mulai 2026, serta rencana penyesuaian target produksi dan porsi domestic market obligation (DMO) batubara yang harganya stagnan sejak 2018. Hal ini memicu diskusi antara pemerintah dan pelaku usaha terkait dampaknya terhadap biaya produksi dan potensi beban pada tarif listrik nasional.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45969</v>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>45975</v>
+      <c r="A4" s="8" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>46005</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1. Harga minyak global menunjukkan kenaikan, dengan Brent di atas USD64 per barel dan West Texas Intermediate di sekitar USD60 per barel, didukung oleh perkembangan positif di Amerika Serikat. Kenaikan ini terjadi setelah harga minyak mentah turun dalam lima dari enam pekan terakhir karena kekhawatiran kelebihan pasokan. Pasar sedang menantikan rilis data pasokan dan permintaan dari OPEC, IEA, dan EIA pekan ini, sementara OPEC dan sekutunya berencana menunda kenaikan produksi pada kuartal pertama tahun depan untuk mengelola pasokan.
-2. Produksi minyak mentah Rusia sedikit meningkat pada Oktober menjadi rata-rata 9.411 mb/d, 43.000 b/d lebih tinggi dari September, namun masih 70.000 b/d di bawah kuota OPEC+ yang mencakup pemotongan kompensasi. Sanksi terbaru Amerika Serikat terhadap sektor energi Rusia, termasuk Rosneft PJSC dan Lukoil PJSC, telah mengurangi ekspor minyak mentah karena beberapa kilang di India, China, dan Turki enggan menerima pasokan yang terkena sanksi.
-3. India, sebagai importir minyak mentah terbesar ketiga di dunia, mengurangi pembelian minyak dari Rusia untuk pengiriman Desember sebagai dampak sanksi Barat dan negosiasi dagang dengan Amerika Serikat. Lima perusahaan kilang besar di India, yang menyumbang sekitar dua pertiga dari total impor minyak Rusia India tahun ini, tidak mengajukan pesanan untuk bulan tersebut. Pergeseran ini mendorong India untuk mencari pasokan alternatif dari kawasan Amerika dan Timur Tengah, mengingat sekitar 36% dari total impor minyak mentah India tahun ini berasal dari Rusia.</t>
-        </is>
-      </c>
+          <t>1.  Upaya transisi energi Indonesia menghadapi tantangan dan perubahan kebijakan, ditandai dengan pembatalan pensiun dini Pembangkit Listrik Tenaga Uap (PLTU) Cirebon-1 yang kemudian pemerintah mencari alternatif pembangkit lain untuk disuntik mati. Selain itu, terdapat kekhawatiran terkait keterlambatan proyek Pembangkit Listrik Tenaga Air (PLTA) dan kritik terhadap target Pembangkit Listrik Tenaga Surya (PLTS) 100 gigawatt. Pemerintah juga menjajaki kerja sama pengembangan Pembangkit Listrik Tenaga Nuklir (PLTN), termasuk tawaran dari Rusia, dengan rencana lelang mitra.
+2.  Pemerintah berencana menerapkan kebijakan fiskal baru seperti bea keluar untuk ekspor batu bara (1%-5%) dan emas (7,5%-15%) mulai tahun 2026 guna mendorong hilirisasi dan meningkatkan penerimaan negara. Selain itu, pemerintah mengkaji pengalihan subsidi LPG untuk mendukung proyek hilirisasi batu bara menjadi Dimethyl Ether (DME) yang ditargetkan mulai konstruksi pada 2026. Kementerian Energi dan Sumber Daya Mineral (ESDM) juga menolak ekspor listrik energi baru terbarukan (EBT) mentah dan mendorong hilirisasi EBT di dalam negeri.
+3.  Sektor ketenagalistrikan di Aceh, Sumatra Utara, dan Sumatra Barat menghadapi kendala berat dalam pemulihan pasokan listrik pasca-bencana banjir dan longsor, yang juga menghambat pemulihan infrastruktur telekomunikasi. Di sisi lain, angkutan batu bara oleh PT Kereta Api Indonesia (Persero) mencatat peningkatan, menunjukkan peran bahan bakar tersebut dalam menopang kebutuhan Pembangkit Listrik Tenaga Uap (PLTU) di Jawa dan Bali.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45976</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>45982</v>
+      <c r="A5" s="8" t="n">
+        <v>46006</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>46012</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1. Indonesia sedang menyiapkan Peraturan Presiden yang memperbolehkan PT Pertamina (Persero) untuk mengimpor energi langsung dari perusahaan Amerika Serikat tanpa proses lelang. Kebijakan ini merupakan tindak lanjut dari kesepakatan tarif timbal balik antara AS dan Indonesia pada Juli 2025, dengan tujuan mengurangi defisit perdagangan AS dengan Indonesia yang sekitar US$18 miliar, dan mengakselerasi komitmen impor minyak Indonesia dari AS senilai US$15 miliar. PT Kilang Pertamina Internasional (KPI) mencari cara agar impor minyak mentah dari AS dapat lebih ekonomis, dan pemerintah berencana meningkatkan impor minyak mentah dari AS mulai Desember 2025.
-2. Harga minyak global terkoreksi di pekan ini, dengan harga berjangka Brent turun US$1,63 (2,5%) menjadi US$63,26 per barel dan West Texas Intermediate (WTI) melemah US$1,56 (2,6%) menjadi US$59,18 per barel pada 20 November 2025. Penurunan ini dipengaruhi oleh laporan upaya AS untuk mengakhiri perang Rusia-Ukraina, yang berpotensi meningkatkan pasokan minyak Rusia ke pasar. Bersamaan dengan itu, sanksi AS terhadap Rosneft dan Lukoil mulai berlaku pada 21 November 2025, berpotensi membuat hampir 48 juta barel minyak mentah Rusia terlantar di laut dan mendorong pembeli di Asia mencari pasokan alternatif.
-3. Harga minyak mentah Indonesia (ICP) untuk Oktober 2025 ditetapkan sebesar US$63,62 per barel, turun US$3,19 per barel dari bulan sebelumnya. Penurunan ini disebabkan oleh beberapa faktor seperti peningkatan suplai minyak oleh OPEC+ sebesar 137.000 barel per hari untuk November 2025, berkurangnya ketegangan geopolitik di Timur Tengah, pengolahan minyak mentah global yang diperkirakan mencapai titik terendah musiman 81,6 juta barel per hari pada Oktober, penguatan nilai tukar dolar AS, serta pemotongan harga jual resmi minyak mentah Arab Saudi untuk pembeli di Asia di tengah melemahnya permintaan dan perlambatan ekonomi Tiongkok.</t>
-        </is>
-      </c>
+          <t>1.  Pemerintah dan PT PLN (Persero) terus berupaya memulihkan pasokan listrik di wilayah Sumatra, terutama Aceh, yang terdampak bencana banjir dan tanah longsor. Pemulihan menghadapi tantangan karena kerusakan infrastruktur yang parah dan area yang terisolasi. Meskipun listrik di Banda Aceh telah pulih, beberapa kabupaten masih mengalami kendala listrik bergilir akibat kerusakan infrastruktur tegangan rendah. Berbagai pihak terlibat dalam penyaluran bantuan dan perbaikan.
+2.  Ekosistem kendaraan listrik di Indonesia menunjukkan perkembangan, ditandai dengan peresmian pabrik baru, penambahan Stasiun Pengisian Kendaraan Listrik Umum (SPKLU) oleh PLN, dan pertumbuhan penjualan kendaraan listrik. Di sisi energi terbarukan, PLN Energi Primer Indonesia menargetkan peningkatan penggunaan biomassa untuk co-firing di PLTU dan mengkaji pengembangan Pembangkit Listrik Tenaga Surya (PLTS) Terapung Cirata. Investasi dalam energi surya semakin kompetitif karena penurunan biaya.
+3.  Pemerintah sedang menyusun kebijakan fiskal di sektor energi, termasuk rencana pengenaan bea keluar untuk ekspor batu bara dan emas mulai Januari 2026 guna menambah penerimaan negara dan menyeimbangkan pasar. Pembahasan mengenai pajak karbon dan kelayakan ekonomi proyek gasifikasi batu bara menjadi Dimethyl Ether (DME) sebagai pengganti LPG juga berlanjut, dengan pertimbangan besar tentang subsidi yang dibutuhkan. Selain itu, pemerintah berencana memperketat aturan pembelian LPG 3 kg.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45983</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>45989</v>
+      <c r="A6" s="8" t="n">
+        <v>46013</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>46019</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.  Harga minyak menunjukkan tekanan turun selama minggu ini, dengan Brent diperdagangkan di kisaran USD 62-63 per barel dan WTI Crude di kisaran USD 58-59 per barel. Prediksi dari bank investasi seperti Goldman Sachs memperkirakan WTI Crude akan rata-rata USD 53 per barel pada 2026, sementara JP Morgan memproyeksikan Brent dapat turun ke kisaran USD 30-an per barel pada 2027 karena kekhawatiran pasokan berlebih sebesar 2 juta barel per hari. Harga bensin eceran di Amerika Serikat turun di bawah USD 3 per galon di banyak negara bagian, dengan beberapa lokasi mencapai USD 1.99 per galon.
-2.  Pasokan minyak global tetap kuat, didorong oleh produksi yang tangguh dari produsen non-OPEC seperti Amerika Serikat, Brasil, dan Guyana. Meskipun eksekutif shale AS melaporkan tantangan profitabilitas di bawah USD 60 per barel dan kenaikan biaya pengeboran sebesar 5 hingga 10 persen dari tahun lalu, produksi shale AS terus meningkat. OPEC+ diperkirakan akan mempertahankan tingkat produksi saat ini pada pertemuan tanggal 30 November, menunda peningkatan produksi yang direncanakan untuk kuartal I 2026 akibat kekhawatiran peningkatan persediaan global.
-3.  Pembicaraan damai yang diperbarui antara Rusia dan Ukraina memberikan tekanan signifikan pada harga minyak karena potensi pelonggaran sanksi yang dapat meningkatkan pasokan Rusia. Di sisi lain, konferensi energi di Timur Tengah menampilkan pandangan yang berbeda, dengan ADIPEC menyoroti permintaan energi jangka panjang yang kuat dan kebutuhan investasi besar USD 18.2 triliun untuk mencapai 123 juta barel per hari pada 2050, sementara Dii Desert Energy Summit berfokus pada percepatan pertumbuhan energi rendah karbon dan investasi yang melampaui bahan bakar fosil dengan rasio 2 berbanding 1. Cina terus mempercepat pembelian minyak mentah strategisnya, mengimpor sekitar 2.15 juta barel per hari dari Rusia dan menimbun lebih dari 1 juta barel per hari pada beberapa bulan di tahun 2025.</t>
-        </is>
-      </c>
+          <t>1. PLN dan mitra strategis terus mempercepat pengembangan energi baru terbarukan (EBT) sesuai Rencana Usaha Penyediaan Tenaga Listrik (RUPTL) 2025–2034, yang menargetkan 76% dari penambahan kapasitas pembangkit berasal dari EBT. Kolaborasi dengan Danantara Investment Management akan menjajaki investasi besar pada proyek-proyek EBT, dan kesepakatan tarif listrik telah dicapai untuk PLTP Ulubelu 30 MW. Selain itu, pemerintah memastikan keberlanjutan operasional PLTSa Benowo melalui alokasi anggaran Rp120 miliar dan Pertamina NRE meluncurkan PLTS di Batam.
+2. Pemerintah tidak akan melanjutkan insentif kendaraan listrik (EV) pada 2026, termasuk pembebasan PPN dan bea masuk impor CBU, yang dapat mempengaruhi pertumbuhan pasar EV. Meskipun demikian, produsen seperti BYD dan VinFast berencana menjaga harga dengan fokus pada produksi lokal. Guna mendukung ekosistem EV, PLN telah menyiagakan lebih dari 4.500 Stasiun Pengisian Kendaraan Listrik Umum (SPKLU) di berbagai wilayah untuk periode Natal dan Tahun Baru, serta PLN bekerja sama dengan KAI untuk elektrifikasi jalur KRL Cikampek.
+3. Mulai 2026, pemerintah akan menerapkan bea keluar pada ekspor batu bara dengan proyeksi penerimaan Rp25 triliun per tahun, sebagai respons terhadap tingginya restitusi Pajak Pertambahan Nilai (PPN) dari sektor batu bara. Sementara itu, PLN terus berupaya memulihkan dan meningkatkan keandalan pasokan listrik di wilayah Aceh, Sumatra Utara, dan Sumatra Barat yang terdampak bencana, termasuk mengoperasikan jalur transmisi kedua Arun–Bireuen dan Pembangkit Listrik Tenaga Gas (PLTG) Tanjung Selor 20 MW di Kalimantan Utara.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45990</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>45991</v>
+      <c r="A7" s="8" t="n">
+        <v>46020</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>46020</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45992</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>45998</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1. OPEC+ menegaskan kembali rencana untuk menahan kenaikan produksi minyak mentah sepanjang kuartal I 2026 di tengah ekspektasi pelemahan pasar musiman dan potensi surplus pasokan global. Badan Energi Internasional (IEA) memproyeksikan rekor kelebihan pasokan pada 2026, sementara harga Brent diperdagangkan mendekati USD63/bbl dan West Texas Intermediate (WTI) mendekati USD59/bbl pada awal Desember 2025.
-2. Ketegangan geopolitik, seperti retorika dan pengerahan pasukan Amerika Serikat di bawah Presiden Donald Trump terkait Venezuela, serta upaya perundingan damai antara Amerika Serikat dan Rusia mengenai konflik Ukraina, terus menopang harga minyak dengan menambah premi risiko. Potensi gencatan senjata di Ukraina dapat membuka peluang pelonggaran sanksi terhadap Rusia dan peningkatan ekspor minyak, yang berpotensi menekan harga lebih lanjut.
-3. Indikasi kelebihan pasokan global tetap menjadi perhatian, didorong oleh lonjakan pasokan dari Amerika dan kenaikan persediaan minyak mentah AS sekitar 574.000 barel pada pekan lalu. Di sisi domestik, PT Pertamina International Shipping (PIS) menyiagakan 332 armada kapal tanker ditambah 12 kapal cadangan untuk memastikan kelancaran distribusi minyak mentah, BBM, LPG, dan petrokimia di Indonesia selama periode Natal 2025 dan Tahun Baru 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45999</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>46005</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1. Harga minyak global menunjukkan volatilitas dan tren bearish menjelang akhir pekan, berfluktuasi antara sekitar US$57–US$64 per barel. Penurunan suku bunga acuan Federal Reserve sebesar 25 basis poin sesuai ekspektasi pasar, namun kekhawatiran kelebihan pasokan global dan perkembangan negosiasi Rusia-Ukraina yang mengarah ke jalur perdamaian menekan harga minyak.
-2. Kekhawatiran kelebihan pasokan global menjadi sentimen dominan, dengan laporan International Energy Agency (IEA) mencatat pasokan minyak dunia mencapai 109 juta barel per hari pada November. IEA merevisi perkiraan surplus global untuk tahun 2026 menjadi 3.84 juta barel per hari, sedikit lebih rendah dari proyeksi sebelumnya, didorong oleh peningkatan proyeksi pertumbuhan permintaan.
-3. Tiongkok terus melakukan penimbunan minyak mentah strategis dan komersial dengan rata-rata sekitar 1 juta barel per hari pada tahun 2025, dan diproyeksikan sekitar 900.000 barel per hari pada tahun 2026, yang membantu meredam kelebihan pasokan di pasar global. Sementara itu, Kementerian Energi dan Sumber Daya Mineral Indonesia melaporkan kerugian devisa negara sebesar Rp523 triliun per tahun karena impor minyak yang mencapai 313 juta barel pada 2024.</t>
-        </is>
-      </c>
+          <t>1. Penggunaan kendaraan listrik di Indonesia menunjukkan peningkatan, tercermin dari lonjakan pengisian daya selama periode Natal dan Tahun Baru 2025/2026, didukung oleh penambahan infrastruktur Stasiun Pengisian Kendaraan Listrik Umum (SPKLU) oleh PLN.
+2. Pemerintah Indonesia sedang membahas insentif untuk mendorong industri kendaraan listrik, khususnya yang berkaitan dengan pemanfaatan sumber daya nikel domestik, meskipun terdapat perdebatan mengenai potensi distorsi teknologi akibat preferensi jenis baterai tertentu.
+3. Sektor energi Indonesia menghadapi tantangan operasional, seperti pemulihan kelistrikan pascabencana di Sumatra, serta dampak fluktuasi harga komoditas batu bara terhadap penerimaan negara.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1903,7 +1908,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -1949,9 +1954,9 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.  OPEC+ mengumumkan penghentian sementara kenaikan produksi pada kuartal I-2026 setelah kenaikan moderat pada Desember, sebagai upaya menyeimbangkan pasar di tengah tanda-tanda kelebihan pasokan. Morgan Stanley menaikkan proyeksi harga Brent menjadi USD60/bbl untuk semester I-2026, namun mencatat peningkatan produksi OPEC+ sebesar 500.000 bph dari Maret hingga Oktober jauh di bawah kenaikan kuota 2,6 mb/d.
-2.  Harga minyak mentah global melemah dan mencatat penurunan mingguan kedua, tertekan oleh peningkatan pasokan dari OPEC+ serta produsen non-anggota seperti Amerika Serikat dan Brasil. Brent turun menjadi sekitar USD63/bbl dan WTI di bawah USD60/bbl, dengan WTI anjlok sekitar 16% hingga 17% sepanjang tahun ini. Data American Petroleum Institute (API) menunjukkan stok minyak mentah Amerika Serikat naik 6,5 juta barel pada pekan lalu.
-3.  Kilang-kilang minyak di China, termasuk milik negara dan swasta, menghentikan pembelian minyak mentah asal Rusia setelah Amerika Serikat menjatuhkan sanksi terhadap produsen utama Moskow, memengaruhi sekitar 400.000 bpd atau hampir 45% dari total impor minyak Rusia ke China. Menanggapi pasar yang cukup mendapat pasokan dan lemahnya permintaan di Asia, Saudi Aramco memangkas harga minyak mentah unggulannya, Arab Light, untuk pasar Asia pada Desember sebesar USD1.20/bbl.</t>
+          <t>1. Harga minyak mentah global mengalami tekanan penurunan sepanjang minggu pertama November 2025 akibat kekhawatiran kelebihan pasokan dan lemahnya permintaan, khususnya dari Amerika Serikat. Harga Brent diperdagangkan di sekitar US$63-US$64 per barel, dan West Texas Intermediate (WTI) mendekati US$60 per barel, dengan WTI anjlok sekitar 16-17% secara tahun berjalan. Stok minyak mentah AS menunjukkan kenaikan signifikan, dengan laporan API sebesar 6.5 juta barel dan EIA sebesar 5.2 juta barel pada pekan lalu.
+2. OPEC+ memutuskan untuk menghentikan sementara rencana kenaikan produksi pada kuartal I 2026, setelah peningkatan moderat pada Desember, sebagai upaya menyeimbangkan pasar dan meredam volatilitas. Morgan Stanley menaikkan proyeksi harga Brent menjadi US$60 per barel untuk semester I 2026 dari US$57.50. Namun, proyeksi tekanan harga tetap ada, dengan Capital Economics memperkirakan Brent mencapai US$60 per barel pada akhir 2025 dan US$50 per barel pada akhir 2026.
+3. Sanksi AS terhadap produsen minyak utama Rusia (Rosneft PJSC dan Lukoil PJSC) mengakibatkan kilang-kilang di China menghentikan pembelian minyak mentah Rusia, mempengaruhi sekitar 400.000 barel per hari atau 45% dari total impor Rusia ke China. Kondisi pasar yang cukup pasokan ini mendorong Arab Saudi untuk memangkas harga jual minyak mentah utamanya untuk pembeli Asia pada Desember, termasuk Arab Light yang dipangkas US$1.20 per barel.</t>
         </is>
       </c>
     </row>
@@ -1964,9 +1969,9 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1. Produksi minyak mentah Rusia pada Oktober mencapai rata-rata 9.411 juta barel per hari, meningkat 43.000 barel per hari dari September. Angka ini 70.000 barel per hari di bawah kuota OPEC+ yang mencakup pemotongan kompensasi, dengan target yang dibutuhkan sebesar 9.481 juta barel per hari. Sanksi terbaru Amerika Serikat terhadap sektor energi Rusia, termasuk Rosneft PJSC dan Lukoil PJSC, telah mengurangi ekspor minyak mentah karena keengganan beberapa kilang di India, China, dan Turki untuk menerima minyak yang terkena sanksi.
-2. Harga minyak global menunjukkan kenaikan, dengan Brent melewati US$64 per barel dan West Texas Intermediate (WTI) bergerak di kisaran US$60 per barel, didorong oleh upaya mengakhiri penutupan pemerintahan Amerika Serikat. Kekhawatiran akan kelebihan pasokan masih membebani pasar, menyebabkan harga minyak mentah turun dalam lima dari enam pekan terakhir. Organisasi Negara-Negara Pengekspor Minyak (OPEC) dan sekutunya mulai melonggarkan pembatasan produksi, namun berencana menunda kenaikan output pada kuartal pertama tahun depan, sementara produsen non-OPEC termasuk Amerika Serikat terus menambah pasokan.
-3. India, importir minyak terbesar ketiga di dunia, mengurangi pembelian minyak mentah dari Rusia untuk pengiriman Desember. Lima perusahaan kilang besar di India, yang menyumbang sekitar dua pertiga dari total impor minyak Rusia tahun ini, belum mengajukan pesanan. Perubahan pola pembelian ini sebagian besar didorong oleh sanksi Barat terhadap produsen minyak Rusia dan negosiasi dagang dengan Amerika Serikat, di mana India berkomitmen membeli lebih banyak minyak mentah dari Amerika Serikat. Akibatnya, kilang-kilang di India mulai mencari alternatif pasokan dari kawasan Amerika dan Timur Tengah, dengan Indian Oil Corp. berupaya membeli hingga 24 juta barel dari Amerika untuk pengiriman Januari hingga Maret.</t>
+          <t>1. Harga minyak global menunjukkan kenaikan, dengan Brent di atas USD64 per barel dan West Texas Intermediate di sekitar USD60 per barel, didukung oleh perkembangan positif di Amerika Serikat. Kenaikan ini terjadi setelah harga minyak mentah turun dalam lima dari enam pekan terakhir karena kekhawatiran kelebihan pasokan. Pasar sedang menantikan rilis data pasokan dan permintaan dari OPEC, IEA, dan EIA pekan ini, sementara OPEC dan sekutunya berencana menunda kenaikan produksi pada kuartal pertama tahun depan untuk mengelola pasokan.
+2. Produksi minyak mentah Rusia sedikit meningkat pada Oktober menjadi rata-rata 9.411 mb/d, 43.000 b/d lebih tinggi dari September, namun masih 70.000 b/d di bawah kuota OPEC+ yang mencakup pemotongan kompensasi. Sanksi terbaru Amerika Serikat terhadap sektor energi Rusia, termasuk Rosneft PJSC dan Lukoil PJSC, telah mengurangi ekspor minyak mentah karena beberapa kilang di India, China, dan Turki enggan menerima pasokan yang terkena sanksi.
+3. India, sebagai importir minyak mentah terbesar ketiga di dunia, mengurangi pembelian minyak dari Rusia untuk pengiriman Desember sebagai dampak sanksi Barat dan negosiasi dagang dengan Amerika Serikat. Lima perusahaan kilang besar di India, yang menyumbang sekitar dua pertiga dari total impor minyak Rusia India tahun ini, tidak mengajukan pesanan untuk bulan tersebut. Pergeseran ini mendorong India untuk mencari pasokan alternatif dari kawasan Amerika dan Timur Tengah, mengingat sekitar 36% dari total impor minyak mentah India tahun ini berasal dari Rusia.</t>
         </is>
       </c>
     </row>
@@ -1979,9 +1984,9 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1. Indonesia berkomitmen untuk meningkatkan impor minyak mentah dari Amerika Serikat hingga US$15 miliar mulai Desember 2025, sebagai bagian dari kesepakatan tarif timbal balik. PT Pertamina (Persero) melalui anak usahanya PT Kilang Pertamina Internasional (KPI) berupaya mencari skema ekonomis untuk impor ini, dengan regulasi baru yang memungkinkan pembelian langsung tanpa lelang dari perusahaan AS.
-2. Harga minyak mentah global mengalami koreksi, dengan Brent turun 2,5% ke US$63,26 per barel dan WTI melemah 2,6% menjadi US$59,18 per barel pada 20 November 2025, dipicu laporan potensi berakhirnya perang Rusia-Ukraina dan peningkatan pasokan OPEC+ sebesar 137.000 barel per hari mulai November 2025. Harga Minyak Mentah Indonesia (ICP) Oktober 2025 ditetapkan US$63,62 per barel, turun US$3,19 per barel dari bulan sebelumnya.
-3. Sanksi Amerika Serikat terhadap produsen minyak Rusia Rosneft PJSC dan Lukoil PJSC yang berlaku pada 21 November 2025 berpotensi menyebabkan hampir 48 juta barel minyak mentah Rusia terlantar di laut, memaksa pembeli di Asia mencari pasokan alternatif dan kapal tanker mencari tujuan baru di tengah tekanan untuk mematuhi sanksi.</t>
+          <t>1. Indonesia sedang menyiapkan Peraturan Presiden yang memperbolehkan PT Pertamina (Persero) untuk mengimpor energi langsung dari perusahaan Amerika Serikat tanpa proses lelang. Kebijakan ini merupakan tindak lanjut dari kesepakatan tarif timbal balik antara AS dan Indonesia pada Juli 2025, dengan tujuan mengurangi defisit perdagangan AS dengan Indonesia yang sekitar US$18 miliar, dan mengakselerasi komitmen impor minyak Indonesia dari AS senilai US$15 miliar. PT Kilang Pertamina Internasional (KPI) mencari cara agar impor minyak mentah dari AS dapat lebih ekonomis, dan pemerintah berencana meningkatkan impor minyak mentah dari AS mulai Desember 2025.
+2. Harga minyak global terkoreksi di pekan ini, dengan harga berjangka Brent turun US$1,63 (2,5%) menjadi US$63,26 per barel dan West Texas Intermediate (WTI) melemah US$1,56 (2,6%) menjadi US$59,18 per barel pada 20 November 2025. Penurunan ini dipengaruhi oleh laporan upaya AS untuk mengakhiri perang Rusia-Ukraina, yang berpotensi meningkatkan pasokan minyak Rusia ke pasar. Bersamaan dengan itu, sanksi AS terhadap Rosneft dan Lukoil mulai berlaku pada 21 November 2025, berpotensi membuat hampir 48 juta barel minyak mentah Rusia terlantar di laut dan mendorong pembeli di Asia mencari pasokan alternatif.
+3. Harga minyak mentah Indonesia (ICP) untuk Oktober 2025 ditetapkan sebesar US$63,62 per barel, turun US$3,19 per barel dari bulan sebelumnya. Penurunan ini disebabkan oleh beberapa faktor seperti peningkatan suplai minyak oleh OPEC+ sebesar 137.000 barel per hari untuk November 2025, berkurangnya ketegangan geopolitik di Timur Tengah, pengolahan minyak mentah global yang diperkirakan mencapai titik terendah musiman 81,6 juta barel per hari pada Oktober, penguatan nilai tukar dolar AS, serta pemotongan harga jual resmi minyak mentah Arab Saudi untuk pembeli di Asia di tengah melemahnya permintaan dan perlambatan ekonomi Tiongkok.</t>
         </is>
       </c>
     </row>
@@ -1994,9 +1999,9 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.  Pada 27 November 2025, harga minyak Brent naik 0.2% menjadi USD 63.34 per barel dan West Texas Intermediate (WTI) menguat 0.8% menjadi USD 59.10 per barel. Kenaikan ini dipicu oleh harapan terobosan pembicaraan perdamaian antara Rusia dan Ukraina, yang menetralkan kekhawatiran pasokan akibat sanksi baru AS terhadap produsen Rusia.
-2.  Organisasi Negara-Negara Pengekspor Minyak dan sekutunya (OPEC+) diperkirakan akan mempertahankan tingkat produksi pada pertemuan mendatang. Selain itu, delapan negara anggota OPEC+ yang secara bertahap meningkatkan produksi pada tahun 2025 diproyeksikan untuk mempertahankan kebijakan jeda kenaikan produksi pada kuartal I 2026.
-3.  Ekspektasi pemangkasan suku bunga acuan oleh The Federal Reserve pada Desember 2025 turut mendorong harga minyak, mengingat penurunan suku bunga dapat mendukung pertumbuhan ekonomi global dan memperkuat permintaan minyak.</t>
+          <t>1.  Harga minyak menunjukkan tekanan turun selama minggu ini, dengan Brent diperdagangkan di kisaran USD 62-63 per barel dan WTI Crude di kisaran USD 58-59 per barel. Prediksi dari bank investasi seperti Goldman Sachs memperkirakan WTI Crude akan rata-rata USD 53 per barel pada 2026, sementara JP Morgan memproyeksikan Brent dapat turun ke kisaran USD 30-an per barel pada 2027 karena kekhawatiran pasokan berlebih sebesar 2 juta barel per hari. Harga bensin eceran di Amerika Serikat turun di bawah USD 3 per galon di banyak negara bagian, dengan beberapa lokasi mencapai USD 1.99 per galon.
+2.  Pasokan minyak global tetap kuat, didorong oleh produksi yang tangguh dari produsen non-OPEC seperti Amerika Serikat, Brasil, dan Guyana. Meskipun eksekutif shale AS melaporkan tantangan profitabilitas di bawah USD 60 per barel dan kenaikan biaya pengeboran sebesar 5 hingga 10 persen dari tahun lalu, produksi shale AS terus meningkat. OPEC+ diperkirakan akan mempertahankan tingkat produksi saat ini pada pertemuan tanggal 30 November, menunda peningkatan produksi yang direncanakan untuk kuartal I 2026 akibat kekhawatiran peningkatan persediaan global.
+3.  Pembicaraan damai yang diperbarui antara Rusia dan Ukraina memberikan tekanan signifikan pada harga minyak karena potensi pelonggaran sanksi yang dapat meningkatkan pasokan Rusia. Di sisi lain, konferensi energi di Timur Tengah menampilkan pandangan yang berbeda, dengan ADIPEC menyoroti permintaan energi jangka panjang yang kuat dan kebutuhan investasi besar USD 18.2 triliun untuk mencapai 123 juta barel per hari pada 2050, sementara Dii Desert Energy Summit berfokus pada percepatan pertumbuhan energi rendah karbon dan investasi yang melampaui bahan bakar fosil dengan rasio 2 berbanding 1. Cina terus mempercepat pembelian minyak mentah strategisnya, mengimpor sekitar 2.15 juta barel per hari dari Rusia dan menimbun lebih dari 1 juta barel per hari pada beberapa bulan di tahun 2025.</t>
         </is>
       </c>
     </row>
@@ -2027,9 +2032,9 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1. PT Pertamina International Shipping (PIS) mengaktifkan Satuan Tugas Nataru 2025/2026 dan menyiagakan 332 kapal tanker utama ditambah 12 kapal cadangan serta 338 kapal pendukung pelabuhan mulai 1 Desember 2025 untuk menjamin kelancaran distribusi minyak mentah, BBM, LPG, dan petrokimia nasional.
-2. Harga minyak dunia menguat pada 1 Desember 2025, dengan Brent diperdagangkan pada US$63 per barel dan West Texas Intermediate (WTI) pada US$59.13 per barel, setelah OPEC+ menegaskan rencana menahan kenaikan produksi sepanjang kuartal I/2026 akibat pelemahan kondisi pasar musiman.
-3. Keputusan OPEC+ untuk mempertahankan jeda pasokan selama tiga bulan diambil di tengah proyeksi surplus pasokan global, dengan Badan Energi Internasional (IEA) memperkirakan rekor kelebihan pasokan pada tahun 2026 dan harga minyak telah merosot 15% sepanjang tahun hingga akhir November 2025.</t>
+          <t>1. OPEC+ menegaskan kembali rencana untuk menahan kenaikan produksi minyak mentah sepanjang kuartal I 2026 di tengah ekspektasi pelemahan pasar musiman dan potensi surplus pasokan global. Badan Energi Internasional (IEA) memproyeksikan rekor kelebihan pasokan pada 2026, sementara harga Brent diperdagangkan mendekati USD63/bbl dan West Texas Intermediate (WTI) mendekati USD59/bbl pada awal Desember 2025.
+2. Ketegangan geopolitik, seperti retorika dan pengerahan pasukan Amerika Serikat di bawah Presiden Donald Trump terkait Venezuela, serta upaya perundingan damai antara Amerika Serikat dan Rusia mengenai konflik Ukraina, terus menopang harga minyak dengan menambah premi risiko. Potensi gencatan senjata di Ukraina dapat membuka peluang pelonggaran sanksi terhadap Rusia dan peningkatan ekspor minyak, yang berpotensi menekan harga lebih lanjut.
+3. Indikasi kelebihan pasokan global tetap menjadi perhatian, didorong oleh lonjakan pasokan dari Amerika dan kenaikan persediaan minyak mentah AS sekitar 574.000 barel pada pekan lalu. Di sisi domestik, PT Pertamina International Shipping (PIS) menyiagakan 332 armada kapal tanker ditambah 12 kapal cadangan untuk memastikan kelancaran distribusi minyak mentah, BBM, LPG, dan petrokimia di Indonesia selama periode Natal 2025 dan Tahun Baru 2026.</t>
         </is>
       </c>
     </row>
@@ -2042,9 +2047,9 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.  Harga minyak global melemah sepanjang minggu dengan Brent diperdagangkan di bawah US$64/bbl dan kemudian turun menjadi US$61,94/bbl, sementara WTI mendekati US$60/bbl dan kemudian merosot ke US$58,25/bbl. Penurunan ini dipicu oleh pemulihan produksi 460.000 barel per hari di ladang minyak West Qurna 2 Irak dan kekhawatiran pasokan global berlebih dari OPEC+, Amerika Serikat, Brasil, dan Guyana. Stok minyak kargo di laut meningkat sekitar 2,5 juta barel per hari sejak pertengahan Agustus.
-2.  Medco Energi menargetkan produksi minyak dan gas bumi mencapai 160.000 barel setara minyak per hari (boepd) pada akhir 2025, meningkat dari 150.000 boepd pada kuartal III/2025, didukung oleh akuisisi 24% Participating Interest di Corridor PSC dan 45% PI di Sakakemang PSC. Perusahaan juga menandatangani perjanjian penjaminan untuk uang muka jual beli transaksi minyak mentah senilai maksimum US$80 juta. Pada semester I/2025, Medco mencatatkan laba bersih US$37,36 juta dari penjualan US$1,13 miliar.
-3.  Perkembangan geopolitik dan makroekonomi memengaruhi pasar minyak, termasuk negosiasi damai Rusia-Ukraina dan serangan terhadap infrastruktur energi Rusia. Negara-negara G7 dan Uni Eropa sedang mempertimbangkan larangan penuh layanan maritim untuk minyak Rusia. China melanjutkan penimbunan minyak mentah dengan perkiraan 800.000 hingga 900.000 barel per hari pada tahun 2026, meskipun pertumbuhan permintaan domestiknya diproyeksikan melambat menjadi 150.000 hingga 320.000 barel per hari pada tahun yang sama. Keputusan suku bunga Federal Reserve AS sebesar 25 basis poin juga dinantikan pasar.</t>
+          <t>1. Harga minyak global menunjukkan volatilitas dan tren bearish menjelang akhir pekan, berfluktuasi antara sekitar US$57–US$64 per barel. Penurunan suku bunga acuan Federal Reserve sebesar 25 basis poin sesuai ekspektasi pasar, namun kekhawatiran kelebihan pasokan global dan perkembangan negosiasi Rusia-Ukraina yang mengarah ke jalur perdamaian menekan harga minyak.
+2. Kekhawatiran kelebihan pasokan global menjadi sentimen dominan, dengan laporan International Energy Agency (IEA) mencatat pasokan minyak dunia mencapai 109 juta barel per hari pada November. IEA merevisi perkiraan surplus global untuk tahun 2026 menjadi 3.84 juta barel per hari, sedikit lebih rendah dari proyeksi sebelumnya, didorong oleh peningkatan proyeksi pertumbuhan permintaan.
+3. Tiongkok terus melakukan penimbunan minyak mentah strategis dan komersial dengan rata-rata sekitar 1 juta barel per hari pada tahun 2025, dan diproyeksikan sekitar 900.000 barel per hari pada tahun 2026, yang membantu meredam kelebihan pasokan di pasar global. Sementara itu, Kementerian Energi dan Sumber Daya Mineral Indonesia melaporkan kerugian devisa negara sebesar Rp523 triliun per tahun karena impor minyak yang mencapai 313 juta barel pada 2024.</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2065,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -2106,9 +2111,9 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1. Pada 1 November 2025, beberapa operator SPBU di Indonesia melakukan penyesuaian harga Bahan Bakar Minyak (BBM). PT Pertamina (Persero) menaikkan harga Dexlite dan Pertamina Dex masing-masing sebesar Rp200 per liter menjadi Rp13.900/liter dan Rp14.200/liter, sementara harga Pertamax, Pertamax Turbo, dan Pertamax Green tetap tidak berubah. SPBU Shell dan BP-AKR mayoritas menurunkan harga produk bensin mereka seperti Shell Super (turun Rp210 menjadi Rp12.680/liter) dan BP 92 (turun Rp210 menjadi Rp12.680/liter), namun menaikkan harga produk diesel mereka.
-2. PT Pertamina Patra Niaga telah menyalurkan 100.000 barel base fuel RON 92 kepada BP-AKR (PT Aneka Petroindo Raya) melalui mekanisme bisnis-ke-bisnis, yang memungkinkan ketersediaan kembali BBM BP 92 di jaringan SPBU BP-AKR. BP-AKR diperkirakan akan membeli tambahan 100.000 barel base fuel lagi yang dijadwalkan tiba pada pekan ketiga November 2025. Kementerian ESDM melaporkan PT Vivo Energy Indonesia juga hampir mencapai kesepakatan untuk pembelian sekitar 100.000 barel base fuel, sedangkan negosiasi dengan Shell Indonesia masih berlangsung.
-3. Menanggapi dugaan masalah kualitas BBM Pertalite yang menyebabkan keluhan kendaraan "brebet" di Jawa Timur, Pertamina Patra Niaga bersama Lemigas Kementerian ESDM telah memeriksa hampir 300 SPBU dan hasil sementara menunjukkan tidak ada kontaminasi air atau etanol. Pertamina juga membuka posko pengaduan dan menyediakan 32 bengkel rekanan untuk perbaikan gratis bagi konsumen yang terdampak. Sementara itu, Kilang Pertamina Internasional (KPI) di Cilacap melanjutkan inisiatif energi hijau, meningkatkan produksi gasoline RON 92 menjadi 53.000 barel per hari dan memproduksi bahan bakar nabati (HVO serta PertaminaSAF).</t>
+          <t>1.  OPEC+ mengumumkan penghentian sementara kenaikan produksi pada kuartal I-2026 setelah kenaikan moderat pada Desember, sebagai upaya menyeimbangkan pasar di tengah tanda-tanda kelebihan pasokan. Morgan Stanley menaikkan proyeksi harga Brent menjadi USD60/bbl untuk semester I-2026, namun mencatat peningkatan produksi OPEC+ sebesar 500.000 bph dari Maret hingga Oktober jauh di bawah kenaikan kuota 2,6 mb/d.
+2.  Harga minyak mentah global melemah dan mencatat penurunan mingguan kedua, tertekan oleh peningkatan pasokan dari OPEC+ serta produsen non-anggota seperti Amerika Serikat dan Brasil. Brent turun menjadi sekitar USD63/bbl dan WTI di bawah USD60/bbl, dengan WTI anjlok sekitar 16% hingga 17% sepanjang tahun ini. Data American Petroleum Institute (API) menunjukkan stok minyak mentah Amerika Serikat naik 6,5 juta barel pada pekan lalu.
+3.  Kilang-kilang minyak di China, termasuk milik negara dan swasta, menghentikan pembelian minyak mentah asal Rusia setelah Amerika Serikat menjatuhkan sanksi terhadap produsen utama Moskow, memengaruhi sekitar 400.000 bpd atau hampir 45% dari total impor minyak Rusia ke China. Menanggapi pasar yang cukup mendapat pasokan dan lemahnya permintaan di Asia, Saudi Aramco memangkas harga minyak mentah unggulannya, Arab Light, untuk pasar Asia pada Desember sebesar USD1.20/bbl.</t>
         </is>
       </c>
     </row>
@@ -2121,9 +2126,9 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1. Pada 10 November 2025, PT Kilang Pertamina Internasional (KPI) memulai pengoperasian awal unit Residual Fluid Catalytic Cracking (RFCC) Complex hasil Proyek Refinery Development Master Plan (RDMP) Balikpapan. Proyek ini akan meningkatkan kapasitas pengolahan minyak mentah dari 260.000 menjadi 360.000 barel per hari, serta memproduksi bahan bakar standar Euro V, tambahan LPG 336.000 ton per tahun, dan propylene 300.000 ton per tahun. Di samping itu, PT Pertamina (Persero) menargetkan keputusan investasi akhir (FID) proyek Kilang Tuban senilai US$24 miliar, dengan kapasitas 300.000 barel per hari, dapat rampung pada awal Desember 2025.
-2. Sepanjang 9-12 November 2025, Kementerian ESDM mendorong pemerataan distribusi BBM dan mengatasi isu pasokan SPBU swasta yang kuota impornya telah habis. BP-AKR telah membeli 100.000 barel base fuel dari Pertamina Patra Niaga dan berencana menambah pembelian 200.000 barel, melalui skema business to business. Sementara itu, Shell dan Vivo masih dalam tahap negosiasi pembelian base fuel dari Pertamina.
-3. Pada 13 November 2025, Kementerian ESDM menyatakan akan mendorong penerapan bensin campuran 10% etanol (E10) pada tahun 2028, dengan kebutuhan etanol diperkirakan mencapai 1,4 juta kiloliter pada 2027. Implementasi E10 menghadapi tantangan seperti ketersediaan bahan baku dan infrastruktur produksi, serta usulan pembebasan etanol bahan bakar dari cukai sebesar Rp20.000 per liter oleh Asosiasi Produsen Spiritus dan Etanol Indonesia (Apsendo) untuk mencegah kenaikan harga produk.</t>
+          <t>1. Produksi minyak mentah Rusia pada Oktober mencapai rata-rata 9.411 juta barel per hari, meningkat 43.000 barel per hari dari September. Angka ini 70.000 barel per hari di bawah kuota OPEC+ yang mencakup pemotongan kompensasi, dengan target yang dibutuhkan sebesar 9.481 juta barel per hari. Sanksi terbaru Amerika Serikat terhadap sektor energi Rusia, termasuk Rosneft PJSC dan Lukoil PJSC, telah mengurangi ekspor minyak mentah karena keengganan beberapa kilang di India, China, dan Turki untuk menerima minyak yang terkena sanksi.
+2. Harga minyak global menunjukkan kenaikan, dengan Brent melewati US$64 per barel dan West Texas Intermediate (WTI) bergerak di kisaran US$60 per barel, didorong oleh upaya mengakhiri penutupan pemerintahan Amerika Serikat. Kekhawatiran akan kelebihan pasokan masih membebani pasar, menyebabkan harga minyak mentah turun dalam lima dari enam pekan terakhir. Organisasi Negara-Negara Pengekspor Minyak (OPEC) dan sekutunya mulai melonggarkan pembatasan produksi, namun berencana menunda kenaikan output pada kuartal pertama tahun depan, sementara produsen non-OPEC termasuk Amerika Serikat terus menambah pasokan.
+3. India, importir minyak terbesar ketiga di dunia, mengurangi pembelian minyak mentah dari Rusia untuk pengiriman Desember. Lima perusahaan kilang besar di India, yang menyumbang sekitar dua pertiga dari total impor minyak Rusia tahun ini, belum mengajukan pesanan. Perubahan pola pembelian ini sebagian besar didorong oleh sanksi Barat terhadap produsen minyak Rusia dan negosiasi dagang dengan Amerika Serikat, di mana India berkomitmen membeli lebih banyak minyak mentah dari Amerika Serikat. Akibatnya, kilang-kilang di India mulai mencari alternatif pasokan dari kawasan Amerika dan Timur Tengah, dengan Indian Oil Corp. berupaya membeli hingga 24 juta barel dari Amerika untuk pengiriman Januari hingga Maret.</t>
         </is>
       </c>
     </row>
@@ -2136,9 +2141,9 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1. Proyek Refinery Development Master Plan Balikpapan menunjukkan kemajuan signifikan dengan pengoperasian awal unit Residual Fluid Catalytic Cracking pada 10 November 2025, menargetkan peresmian pada pertengahan Desember 2025. Investasi sebesar US$7.4 miliar (Rp126 triliun) ini akan meningkatkan kapasitas produksi menjadi 360.000 barel per hari, memenuhi 22-25% kebutuhan energi nasional, dan memangkas ketergantungan impor bahan bakar minyak (BBM) sebesar 10-15% serta avtur mulai tahun 2026. Kilang ini juga akan menghasilkan produk berstandar Euro V dan petrokimia bernilai tinggi.
-2. Pertamina Patra Niaga mencatat peningkatan signifikan pada penjualan produk non-subsidi hingga Oktober 2025, dengan Pertamax Turbo naik 76% secara tahunan dan Pertamax Green 95 naik 80% dibandingkan 2024, yang menyebabkan Pertamina harus menambah pasokan Pertamax Turbo melalui produksi kilang dan impor. Sementara itu, penyaluran BBM bersubsidi seperti Pertalite dan Solar terkendali di bawah kuota masing-masing 10% dan 1.5% dari target 2025, menunjukkan pergeseran konsumen ke BBM beroktan lebih tinggi dan potensi penghematan kompensasi sebesar Rp12.61 triliun.
-3. Harga minyak mentah global mengalami penurunan dengan West Texas Intermediate (WTI) diperdagangkan di atas US$59 per barel dan Brent di bawah US$64 per barel, didorong oleh kenaikan persediaan bensin dan distillate di Amerika Serikat. Di sisi lain, sanksi Amerika Serikat terhadap produsen minyak Rusia dan Iran menghambat aliran minyak mentah ke China dan India, meskipun ketersediaan BBM nasional dipastikan aman dengan cadangan 18-19 hari. Untuk memenuhi permintaan domestik, operator SPBU BP-AKR juga mengandalkan pasokan base fuel dari Pertamina Patra Niaga.</t>
+          <t>1. Indonesia berkomitmen untuk meningkatkan impor minyak mentah dari Amerika Serikat hingga US$15 miliar mulai Desember 2025, sebagai bagian dari kesepakatan tarif timbal balik. PT Pertamina (Persero) melalui anak usahanya PT Kilang Pertamina Internasional (KPI) berupaya mencari skema ekonomis untuk impor ini, dengan regulasi baru yang memungkinkan pembelian langsung tanpa lelang dari perusahaan AS.
+2. Harga minyak mentah global mengalami koreksi, dengan Brent turun 2,5% ke US$63,26 per barel dan WTI melemah 2,6% menjadi US$59,18 per barel pada 20 November 2025, dipicu laporan potensi berakhirnya perang Rusia-Ukraina dan peningkatan pasokan OPEC+ sebesar 137.000 barel per hari mulai November 2025. Harga Minyak Mentah Indonesia (ICP) Oktober 2025 ditetapkan US$63,62 per barel, turun US$3,19 per barel dari bulan sebelumnya.
+3. Sanksi Amerika Serikat terhadap produsen minyak Rusia Rosneft PJSC dan Lukoil PJSC yang berlaku pada 21 November 2025 berpotensi menyebabkan hampir 48 juta barel minyak mentah Rusia terlantar di laut, memaksa pembeli di Asia mencari pasokan alternatif dan kapal tanker mencari tujuan baru di tengah tekanan untuk mematuhi sanksi.</t>
         </is>
       </c>
     </row>
@@ -2151,9 +2156,9 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1. PT Pertamina (Persero) dan anak usahanya, PT Pertamina Patra Niaga (PPN), memperkuat pasokan dan distribusi bahan bakar minyak (BBM) serta LPG menjelang libur Natal 2025 dan Tahun Baru 2026 (Nataru), dengan proyeksi kenaikan konsumsi gasoline 2.3% dan LPG 3.3%. PPN menambah 1.4 juta kiloliter (kl) Pertalite dan memastikan ketahanan stok nasional BBM rata-rata 20.2 hari. Selain itu, stok BBM di SPBU swasta seperti Vivo, BP-AKR, dan Shell secara bertahap kembali tersedia mulai 23 November 2025, setelah membeli base fuel dari PPN. Vivo dan BP-AKR menyerap total 100.000 barel dan 230.000 barel base fuel, sementara Shell telah menyepakati pembelian 100.000 barel base fuel dari PPN.
-2. Pemerintah RI mulai menerapkan skema pembayaran dana kompensasi BBM bersubsidi secara bulanan (70% per bulan) kepada Pertamina efektif 19 November 2025, menggantikan pola kuartalan, yang diperkirakan akan memperkuat likuiditas Pertamina. BPH Migas merencanakan revisi Perpres Nomor 191 Tahun 2014 untuk mengatur tata kelola penjualan Pertalite agar lebih tepat sasaran. Pertamina Patra Niaga juga mempertimbangkan peluang impor Pertalite dari Amerika Serikat sebagai bagian dari strategi pengadaan, menunggu arahan pemerintah.
-3. PT Kilang Pertamina Internasional (KPI) Unit Balikpapan memulai pengoperasian awal unit Residual Fluid Catalytic Cracking (RFCC) berkapasitas 90 ribu barel per hari pada 10 November 2025, bertujuan meningkatkan produksi produk bernilai tinggi dan mengurangi impor BBM. Selain itu, PT AGPA Refinery Complex (ARC) berkapasitas 500.000 ton per tahun di Balikpapan diresmikan pada 21 November 2025 sebagai fasilitas hilir sawit nasional baru, mendukung transformasi energi terbarukan berbasis kelapa sawit. Upaya menjaga operasional kilang Pertamina sebagai objek vital nasional diperkuat dengan pengerahan personel TNI dan BAIS mulai Desember 2025.</t>
+          <t>1.  Pada 27 November 2025, harga minyak Brent naik 0.2% menjadi USD 63.34 per barel dan West Texas Intermediate (WTI) menguat 0.8% menjadi USD 59.10 per barel. Kenaikan ini dipicu oleh harapan terobosan pembicaraan perdamaian antara Rusia dan Ukraina, yang menetralkan kekhawatiran pasokan akibat sanksi baru AS terhadap produsen Rusia.
+2.  Organisasi Negara-Negara Pengekspor Minyak dan sekutunya (OPEC+) diperkirakan akan mempertahankan tingkat produksi pada pertemuan mendatang. Selain itu, delapan negara anggota OPEC+ yang secara bertahap meningkatkan produksi pada tahun 2025 diproyeksikan untuk mempertahankan kebijakan jeda kenaikan produksi pada kuartal I 2026.
+3.  Ekspektasi pemangkasan suku bunga acuan oleh The Federal Reserve pada Desember 2025 turut mendorong harga minyak, mengingat penurunan suku bunga dapat mendukung pertumbuhan ekonomi global dan memperkuat permintaan minyak.</t>
         </is>
       </c>
     </row>
@@ -2184,9 +2189,9 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.  Pertamina Patra Niaga dan operator SPBU swasta seperti Shell, BP, serta Vivo menyesuaikan harga produk kilang nonsubsidi mereka per 1 Desember 2025, yang secara kompak mengalami kenaikan mengacu pada formula harga pemerintah dan tren harga minyak dunia. Namun, khusus tiga wilayah terdampak bencana di Aceh, Sumatra Utara, dan Sumatra Barat, harga BBM nonsubsidi relatif tidak mengalami penyesuaian signifikan. Terkait kinerja ekspor, Badan Pusat Statistik mencatat nilai ekspor Indonesia pada Oktober 2025 mencapai US$24,24 miliar, turun 2,31% dibanding tahun sebelumnya, terutama disebabkan oleh penurunan ekspor bahan bakar mineral sebesar 19,04% nilai dan 7,26% volume.
-2.  Pemerintah dan Pertamina Group mengintensifkan upaya penyaluran dan distribusi energi untuk wilayah Sumatra yang terdampak bencana banjir dan longsor di Aceh, Sumatra Utara, dan Sumatra Barat, serta dalam rangka persiapan periode Natal 2025 dan Tahun Baru 2026 (Nataru). Langkah-langkah yang diambil meliputi pengerahan armada tanker oleh PTPertamina International Shipping, penggunaan moda transportasi beragam seperti pesawat Hercules dan perintis untuk pengiriman BBM ke daerah terisolasi, serta peniadaan sementara sistem barcode MyPertamina untuk pembelian BBM subsidi di daerah bencana. Pertamina Patra Niaga juga berhasil menyuplai total 430.000 barel base fuel kepada SPBU swasta (Shell, BP-AKR, Vivo) untuk menormalisasi kembali ketersediaan BBM mereka.
-3.  Dalam pengembangan industri kilang, PT Kilang Pertamina Internasional (KPI) berkomitmen meningkatkan produksi petrokimia, dengan proyek Refinery Development Master Plan Balikpapan yang akan menghasilkan propilena sekitar 225.000 ton per tahun untuk mengurangi ketergantungan impor. Selain itu, pemerintah berencana merombak skema subsidi energi (BBM dan listrik) dalam dua tahun ke depan untuk meningkatkan efisiensi dan ketepatan sasaran. Pertamina Patra Niaga juga mempertimbangkan opsi impor Pertalite dari Amerika Serikat yang direncanakan mencapai 40% dari total pengadaan, sebagai bagian dari strategi ketahanan energi nasional.</t>
+          <t>1. PT Pertamina International Shipping (PIS) mengaktifkan Satuan Tugas Nataru 2025/2026 dan menyiagakan 332 kapal tanker utama ditambah 12 kapal cadangan serta 338 kapal pendukung pelabuhan mulai 1 Desember 2025 untuk menjamin kelancaran distribusi minyak mentah, BBM, LPG, dan petrokimia nasional.
+2. Harga minyak dunia menguat pada 1 Desember 2025, dengan Brent diperdagangkan pada US$63 per barel dan West Texas Intermediate (WTI) pada US$59.13 per barel, setelah OPEC+ menegaskan rencana menahan kenaikan produksi sepanjang kuartal I/2026 akibat pelemahan kondisi pasar musiman.
+3. Keputusan OPEC+ untuk mempertahankan jeda pasokan selama tiga bulan diambil di tengah proyeksi surplus pasokan global, dengan Badan Energi Internasional (IEA) memperkirakan rekor kelebihan pasokan pada tahun 2026 dan harga minyak telah merosot 15% sepanjang tahun hingga akhir November 2025.</t>
         </is>
       </c>
     </row>
@@ -2199,9 +2204,9 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1. Kementerian Energi dan Sumber Daya Mineral (ESDM) melaporkan devisa negara hilang Rp523 triliun per tahun akibat impor minyak dan Bahan Bakar Minyak (BBM), dengan produksi minyak Indonesia 221 juta barel pada 2024 berbanding impor 313 juta barel. Sebagai upaya penahanan laju impor, Pertamina Patra Niaga telah menyalurkan 430.000 barel base fuel kepada SPBU swasta, mengakhiri kekosongan stok sejak akhir Agustus 2025. Kementerian ESDM juga akan memutuskan kuota impor BBM untuk SPBU swasta pada tahun 2026.
-2. Pertamina Patra Niaga menaikkan harga BBM nonsubsidi per 1 Desember 2025, seperti Pertamax (RON 92) menjadi Rp12.750 per liter dari sebelumnya Rp12.200 per liter, sejalan dengan tren harga minyak global dan nilai tukar rupiah terhadap dolar Amerika Serikat. SPBU swasta juga melakukan penyesuaian harga serupa. Untuk periode Natal 2025 dan Tahun Baru 2026 (Nataru), Pertamina Patra Niaga memproyeksikan kenaikan kebutuhan gasolin 5% dan avtur 1,6%, serta memberikan diskon avtur rata-rata 10% di 37 bandara strategis mulai 22 Desember 2025.
-3. Kilang Pertamina Internasional (KPI) mempercepat proyek Refinery Development Master Plan (RDMP) Balikpapan untuk meningkatkan kapasitas pengolahan minyak mentah dari 260.000 barel menjadi 360.000 barel per hari, dengan target operasi komersial pada 17 Desember 2025. Proyek ini bernilai US$7,4 miliar. Sementara itu, keputusan investasi akhir (FID) untuk proyek Grass Root Refinery (GRR) Kilang Tuban, yang bernilai US$20,7 miliar hingga US$24 miliar, diharapkan diputuskan antara Pertamina dan Rosneft Singapore Pte Ltd pada pertengahan Desember 2025.</t>
+          <t>1.  Harga minyak global melemah sepanjang minggu dengan Brent diperdagangkan di bawah US$64/bbl dan kemudian turun menjadi US$61,94/bbl, sementara WTI mendekati US$60/bbl dan kemudian merosot ke US$58,25/bbl. Penurunan ini dipicu oleh pemulihan produksi 460.000 barel per hari di ladang minyak West Qurna 2 Irak dan kekhawatiran pasokan global berlebih dari OPEC+, Amerika Serikat, Brasil, dan Guyana. Stok minyak kargo di laut meningkat sekitar 2,5 juta barel per hari sejak pertengahan Agustus.
+2.  Medco Energi menargetkan produksi minyak dan gas bumi mencapai 160.000 barel setara minyak per hari (boepd) pada akhir 2025, meningkat dari 150.000 boepd pada kuartal III/2025, didukung oleh akuisisi 24% Participating Interest di Corridor PSC dan 45% PI di Sakakemang PSC. Perusahaan juga menandatangani perjanjian penjaminan untuk uang muka jual beli transaksi minyak mentah senilai maksimum US$80 juta. Pada semester I/2025, Medco mencatatkan laba bersih US$37,36 juta dari penjualan US$1,13 miliar.
+3.  Perkembangan geopolitik dan makroekonomi memengaruhi pasar minyak, termasuk negosiasi damai Rusia-Ukraina dan serangan terhadap infrastruktur energi Rusia. Negara-negara G7 dan Uni Eropa sedang mempertimbangkan larangan penuh layanan maritim untuk minyak Rusia. China melanjutkan penimbunan minyak mentah dengan perkiraan 800.000 hingga 900.000 barel per hari pada tahun 2026, meskipun pertumbuhan permintaan domestiknya diproyeksikan melambat menjadi 150.000 hingga 320.000 barel per hari pada tahun yang sama. Keputusan suku bunga Federal Reserve AS sebesar 25 basis poin juga dinantikan pasar.</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2222,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -2263,9 +2268,9 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1. PT Pertamina Patra Niaga (PPN) menyalurkan 100.000 barel bahan bakar dasar impor kepada BP-AKR untuk menormalisasi pasokan BBM di SPBU swasta, dengan 100.000 barel tambahan diperkirakan tiba pada pekan ketiga November 2025. Badan usaha swasta lainnya, termasuk Vivo dan Shell, masih dalam tahap negosiasi untuk pembelian bahan bakar dasar dari Pertamina.
-2. Per 01 November 2025, Pertamina menaikkan harga Dexlite dan Pertamina Dex sebesar Rp200 per liter, menjadi Rp13.900 per liter dan Rp14.200 per liter. Pada periode yang sama, Shell dan BP-AKR juga menyesuaikan harga BBM, dengan mayoritas jenis bensin turun dan jenis diesel naik.
-3. Terkait dugaan masalah kualitas Pertalite di Jawa Timur, Pertamina Patra Niaga bersama Lemigas Kementerian ESDM melakukan pengecekan di sekitar 300 SPBU. Hasil sementara menunjukkan bahwa Pertalite yang disalurkan "on specification" tanpa kontaminasi air atau etanol, dan Pertamina telah membuka 32 posko pengaduan serta bengkel rekanan untuk memberikan solusi dan kompensasi kepada masyarakat yang terdampak.</t>
+          <t>1. Pada 1 November 2025, beberapa operator SPBU di Indonesia melakukan penyesuaian harga Bahan Bakar Minyak (BBM). PT Pertamina (Persero) menaikkan harga Dexlite dan Pertamina Dex masing-masing sebesar Rp200 per liter menjadi Rp13.900/liter dan Rp14.200/liter, sementara harga Pertamax, Pertamax Turbo, dan Pertamax Green tetap tidak berubah. SPBU Shell dan BP-AKR mayoritas menurunkan harga produk bensin mereka seperti Shell Super (turun Rp210 menjadi Rp12.680/liter) dan BP 92 (turun Rp210 menjadi Rp12.680/liter), namun menaikkan harga produk diesel mereka.
+2. PT Pertamina Patra Niaga telah menyalurkan 100.000 barel base fuel RON 92 kepada BP-AKR (PT Aneka Petroindo Raya) melalui mekanisme bisnis-ke-bisnis, yang memungkinkan ketersediaan kembali BBM BP 92 di jaringan SPBU BP-AKR. BP-AKR diperkirakan akan membeli tambahan 100.000 barel base fuel lagi yang dijadwalkan tiba pada pekan ketiga November 2025. Kementerian ESDM melaporkan PT Vivo Energy Indonesia juga hampir mencapai kesepakatan untuk pembelian sekitar 100.000 barel base fuel, sedangkan negosiasi dengan Shell Indonesia masih berlangsung.
+3. Menanggapi dugaan masalah kualitas BBM Pertalite yang menyebabkan keluhan kendaraan "brebet" di Jawa Timur, Pertamina Patra Niaga bersama Lemigas Kementerian ESDM telah memeriksa hampir 300 SPBU dan hasil sementara menunjukkan tidak ada kontaminasi air atau etanol. Pertamina juga membuka posko pengaduan dan menyediakan 32 bengkel rekanan untuk perbaikan gratis bagi konsumen yang terdampak. Sementara itu, Kilang Pertamina Internasional (KPI) di Cilacap melanjutkan inisiatif energi hijau, meningkatkan produksi gasoline RON 92 menjadi 53.000 barel per hari dan memproduksi bahan bakar nabati (HVO serta PertaminaSAF).</t>
         </is>
       </c>
     </row>
@@ -2278,9 +2283,9 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.  Pemerintah daerah Sumatra Barat dan Pertamina Patra Niaga telah mengambil langkah cepat untuk memulihkan kelangkaan bahan bakar minyak di wilayah tersebut pada November 2025, dengan Pertamina mempercepat pasokan melalui jalur darat dan mengoperasikan Integrated Terminal Teluk Kabung 24 jam sehari sejak 7 November 2025, yang meningkatkan kecepatan penyaluran sekitar 16%. Di sisi lain, Kementerian Energi dan Sumber Daya Mineral mendorong SPBU swasta untuk membeli base fuel dari Pertamina Patra Niaga untuk mengatasi ketimpangan pasokan, di mana BP-AKR telah sepakat membeli dua kargo atau 200.000 barel base fuel, dengan indikasi akan menambah pesanan hingga 300.000 barel, sementara Shell dan Vivo masih dalam tahap negosiasi.
-2.  Kementerian Keuangan mengawal penyelesaian Proyek Refinery Development Master Plan (RDMP) Balikpapan yang ditargetkan meningkatkan kapasitas produksi bahan bakar minyak hingga 142.000 barel per hari, LPG 336.000 ton per tahun, dan propylene 300.000 ton per tahun, dengan nilai investasi mencapai US$7,4 miliar. PT Kilang Pertamina Internasional telah melakukan pengoperasian awal Unit Residual Fluid Catalytic Cracking Complex di RDMP Balikpapan pada 10 November 2025, yang berhasil meningkatkan kapasitas pengolahan minyak mentah dari 260.000 menjadi 360.000 barel per hari dan produksi LPG menjadi 43.000 ton per tahun. Sementara itu, keputusan investasi akhir atau Final Investment Decision (FID) proyek Kilang Tuban berkapasitas 300.000 barel per hari dengan Rosneft ditargetkan rampung pada awal Desember 2025.
-3.  Kementerian Energi dan Sumber Daya Mineral mendorong penerapan bensin campuran 10% etanol (E10) pada 2028, atau berpotensi dipercepat menjadi 2027, dengan kebutuhan etanol mencapai 1,4 juta hingga 4 juta kiloliter. Proyek ini menghadapi tantangan seperti ketersediaan bahan baku, keterbatasan insentif, dan infrastruktur distribusi yang belum memadai, serta usulan dari Asosiasi Produsen Spiritus dan Etanol Indonesia untuk membebaskan etanol dari kategori barang kena cukai sebesar Rp20.000 per liter agar tidak membebani harga bensin hijau bagi konsumen. Pemerintah juga mencari keterlibatan sektor swasta, dengan Toyota Indonesia menunjukkan minat untuk mengembangkan pabrik bioetanol.</t>
+          <t>1. Pada 10 November 2025, PT Kilang Pertamina Internasional (KPI) memulai pengoperasian awal unit Residual Fluid Catalytic Cracking (RFCC) Complex hasil Proyek Refinery Development Master Plan (RDMP) Balikpapan. Proyek ini akan meningkatkan kapasitas pengolahan minyak mentah dari 260.000 menjadi 360.000 barel per hari, serta memproduksi bahan bakar standar Euro V, tambahan LPG 336.000 ton per tahun, dan propylene 300.000 ton per tahun. Di samping itu, PT Pertamina (Persero) menargetkan keputusan investasi akhir (FID) proyek Kilang Tuban senilai US$24 miliar, dengan kapasitas 300.000 barel per hari, dapat rampung pada awal Desember 2025.
+2. Sepanjang 9-12 November 2025, Kementerian ESDM mendorong pemerataan distribusi BBM dan mengatasi isu pasokan SPBU swasta yang kuota impornya telah habis. BP-AKR telah membeli 100.000 barel base fuel dari Pertamina Patra Niaga dan berencana menambah pembelian 200.000 barel, melalui skema business to business. Sementara itu, Shell dan Vivo masih dalam tahap negosiasi pembelian base fuel dari Pertamina.
+3. Pada 13 November 2025, Kementerian ESDM menyatakan akan mendorong penerapan bensin campuran 10% etanol (E10) pada tahun 2028, dengan kebutuhan etanol diperkirakan mencapai 1,4 juta kiloliter pada 2027. Implementasi E10 menghadapi tantangan seperti ketersediaan bahan baku dan infrastruktur produksi, serta usulan pembebasan etanol bahan bakar dari cukai sebesar Rp20.000 per liter oleh Asosiasi Produsen Spiritus dan Etanol Indonesia (Apsendo) untuk mencegah kenaikan harga produk.</t>
         </is>
       </c>
     </row>
@@ -2293,9 +2298,9 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.  Penyelesaian Proyek Refinery Development Master Plan (RDMP) Balikpapan senilai 7.4 miliar USD ditargetkan pada pertengahan Desember 2025. Proyek ini akan meningkatkan kapasitas kilang dari 260.000 barel per hari (bph) menjadi 360.000 bph, berpotensi mengurangi ketergantungan impor Bahan Bakar Minyak (BBM) hingga 15% dan memenuhi 22%-25% kebutuhan energi domestik. Unit Residual Fluid Catalytic Cracking (RFCC) Complex dengan kapasitas 90.000 bph telah mulai beroperasi pada 10 November 2025.
-2.  PT Pertamina Patra Niaga mencatat volume penjualan bensin dan solar sebesar 87 juta kiloliter (KL) per Oktober 2025, dengan 41% berasal dari produk non-subsidi. Penyaluran Solar bersubsidi terkendali 1.5% di bawah kuota 18.8 juta KL dan Pertalite 10% di bawah kuota 31.2 juta KL hingga Oktober 2025. Permintaan Pertamax Turbo (RON 98) melonjak 76%, sehingga Pertamina menambah pasokan melalui impor dan memastikan kesiapan distribusi untuk periode Natal dan Tahun Baru 2025-2026.
-3.  Dalam pengembangan biofuel, penjualan Pertamax Green 95 (E5) di 168 SPBU Pertamina mencatat pertumbuhan 80% dari 2024, dengan proyeksi kebutuhan bioetanol 4,800-5,000 KL per tahun untuk Pulau Jawa. Asosiasi Produsen Spiritus dan Etanol Indonesia (Aspendo) mengusulkan penghapusan cukai bioetanol fuel grade sebesar Rp20.000 per liter untuk menjaga harga kompetitif. Sementara itu, BP-AKR membeli 100.000 barel base fuel dari Pertamina Patra Niaga untuk mengatasi kekurangan stok, sedangkan Shell dan Vivo masih dalam negosiasi business-to-business untuk pengadaan base fuel.</t>
+          <t>1. Proyek Refinery Development Master Plan Balikpapan menunjukkan kemajuan signifikan dengan pengoperasian awal unit Residual Fluid Catalytic Cracking pada 10 November 2025, menargetkan peresmian pada pertengahan Desember 2025. Investasi sebesar US$7.4 miliar (Rp126 triliun) ini akan meningkatkan kapasitas produksi menjadi 360.000 barel per hari, memenuhi 22-25% kebutuhan energi nasional, dan memangkas ketergantungan impor bahan bakar minyak (BBM) sebesar 10-15% serta avtur mulai tahun 2026. Kilang ini juga akan menghasilkan produk berstandar Euro V dan petrokimia bernilai tinggi.
+2. Pertamina Patra Niaga mencatat peningkatan signifikan pada penjualan produk non-subsidi hingga Oktober 2025, dengan Pertamax Turbo naik 76% secara tahunan dan Pertamax Green 95 naik 80% dibandingkan 2024, yang menyebabkan Pertamina harus menambah pasokan Pertamax Turbo melalui produksi kilang dan impor. Sementara itu, penyaluran BBM bersubsidi seperti Pertalite dan Solar terkendali di bawah kuota masing-masing 10% dan 1.5% dari target 2025, menunjukkan pergeseran konsumen ke BBM beroktan lebih tinggi dan potensi penghematan kompensasi sebesar Rp12.61 triliun.
+3. Harga minyak mentah global mengalami penurunan dengan West Texas Intermediate (WTI) diperdagangkan di atas US$59 per barel dan Brent di bawah US$64 per barel, didorong oleh kenaikan persediaan bensin dan distillate di Amerika Serikat. Di sisi lain, sanksi Amerika Serikat terhadap produsen minyak Rusia dan Iran menghambat aliran minyak mentah ke China dan India, meskipun ketersediaan BBM nasional dipastikan aman dengan cadangan 18-19 hari. Untuk memenuhi permintaan domestik, operator SPBU BP-AKR juga mengandalkan pasokan base fuel dari Pertamina Patra Niaga.</t>
         </is>
       </c>
     </row>
@@ -2308,9 +2313,9 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1. PT Pertamina Patra Niaga memperkuat pasokan BBM untuk periode Natal 2025 dan Tahun Baru 2026. Ini mencakup penambahan 1,4 juta kiloliter Pertalite dari produksi kilang domestik dan impor baru, dengan target ketahanan stok 21-23 hari per 25 November 2025. Kilang Pertamina Internasional juga memulai operasi awal unit Residual Fluid Catalytic Cracking (RFCC) berkapasitas 90 ribu barel per hari di Kilang Balikpapan sejak 10 November 2025, yang akan meningkatkan produksi gasoline dan LPG serta mengurangi impor.
-2. Pasokan BBM di SPBU swasta mulai normal kembali setelah mencapai kesepakatan pembelian base fuel dari Pertamina Patra Niaga. Vivo Energy Indonesia telah menerima 100.000 barel Revvo 92 (RON 92) yang mulai tersedia bertahap sejak 23 November 2025. BP-AKR menambah pembelian base fuel menjadi total 230.000 barel dari Pertamina Patra Niaga per 27 November 2025. Shell Indonesia juga menyelesaikan kesepakatan pada 25 November 2025 untuk membeli 100.000 barel base fuel, dengan harapan stok pulih akhir November 2025.
-3. Distribusi energi menghadapi tantangan cuaca ekstrem dan diperkuat dengan langkah keamanan. Dua kapal pengangkut Pertalite dan Biosolar tidak dapat bersandar di Belawan, Sumatra Utara sejak 23 November 2025 karena cuaca ekstrem, menyebabkan penyesuaian pola suplai dari terminal alternatif. Untuk mengamankan infrastruktur energi nasional, pemerintah akan mengerahkan personel TNI untuk menjaga kilang minyak dan terminal BBM Pertamina yang memiliki kapasitas pengolahan 1 juta barel per hari dan 231 terminal migas, dimulai pada Desember 2025.</t>
+          <t>1. PT Pertamina (Persero) dan anak usahanya, PT Pertamina Patra Niaga (PPN), memperkuat pasokan dan distribusi bahan bakar minyak (BBM) serta LPG menjelang libur Natal 2025 dan Tahun Baru 2026 (Nataru), dengan proyeksi kenaikan konsumsi gasoline 2.3% dan LPG 3.3%. PPN menambah 1.4 juta kiloliter (kl) Pertalite dan memastikan ketahanan stok nasional BBM rata-rata 20.2 hari. Selain itu, stok BBM di SPBU swasta seperti Vivo, BP-AKR, dan Shell secara bertahap kembali tersedia mulai 23 November 2025, setelah membeli base fuel dari PPN. Vivo dan BP-AKR menyerap total 100.000 barel dan 230.000 barel base fuel, sementara Shell telah menyepakati pembelian 100.000 barel base fuel dari PPN.
+2. Pemerintah RI mulai menerapkan skema pembayaran dana kompensasi BBM bersubsidi secara bulanan (70% per bulan) kepada Pertamina efektif 19 November 2025, menggantikan pola kuartalan, yang diperkirakan akan memperkuat likuiditas Pertamina. BPH Migas merencanakan revisi Perpres Nomor 191 Tahun 2014 untuk mengatur tata kelola penjualan Pertalite agar lebih tepat sasaran. Pertamina Patra Niaga juga mempertimbangkan peluang impor Pertalite dari Amerika Serikat sebagai bagian dari strategi pengadaan, menunggu arahan pemerintah.
+3. PT Kilang Pertamina Internasional (KPI) Unit Balikpapan memulai pengoperasian awal unit Residual Fluid Catalytic Cracking (RFCC) berkapasitas 90 ribu barel per hari pada 10 November 2025, bertujuan meningkatkan produksi produk bernilai tinggi dan mengurangi impor BBM. Selain itu, PT AGPA Refinery Complex (ARC) berkapasitas 500.000 ton per tahun di Balikpapan diresmikan pada 21 November 2025 sebagai fasilitas hilir sawit nasional baru, mendukung transformasi energi terbarukan berbasis kelapa sawit. Upaya menjaga operasional kilang Pertamina sebagai objek vital nasional diperkuat dengan pengerahan personel TNI dan BAIS mulai Desember 2025.</t>
         </is>
       </c>
     </row>
@@ -2341,9 +2346,9 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1. Kilang Pertamina Internasional (KPI) menargetkan produksi untuk November 2025 sebesar 8 juta barel gasoline, 10,7 juta barel gasoil, dan 2,2 juta barel avtur. Untuk Desember 2025, produksi gasoil seri ditingkatkan menjadi sekitar 11,5 juta barel, sementara volume gasoline dan avtur dipertahankan sesuai rencana November 2025 guna mendukung kelancaran pasokan BBM menjelang periode Natal dan Tahun Baru 2026.
-2. Badan Pusat Statistik (BPS) mencatat volume ekspor bahan bakar mineral (BBM) Indonesia turun sebesar 7,26% pada Oktober 2025 dibandingkan periode yang sama tahun lalu. Penurunan ini merupakan bagian dari total ekspor migas yang turun 33,60% secara tahunan menjadi US$0,89 miliar.
-3. PT Pertamina Patra Niaga (PPN) memasok total 430.000 barel base fuel kepada badan usaha SPBU swasta seperti Shell, Vivo, dan BP-AKR untuk memastikan ketersediaan BBM. PPN juga memproyeksikan peningkatan konsumsi gasoline sebesar 8,4% dan avtur sebesar 2,4% selama periode Nataru 2025/2026 di wilayah Jawa Timur, Bali, dan Nusa Tenggara.</t>
+          <t>1.  Pertamina Patra Niaga dan operator SPBU swasta seperti Shell, BP, serta Vivo menyesuaikan harga produk kilang nonsubsidi mereka per 1 Desember 2025, yang secara kompak mengalami kenaikan mengacu pada formula harga pemerintah dan tren harga minyak dunia. Namun, khusus tiga wilayah terdampak bencana di Aceh, Sumatra Utara, dan Sumatra Barat, harga BBM nonsubsidi relatif tidak mengalami penyesuaian signifikan. Terkait kinerja ekspor, Badan Pusat Statistik mencatat nilai ekspor Indonesia pada Oktober 2025 mencapai US$24,24 miliar, turun 2,31% dibanding tahun sebelumnya, terutama disebabkan oleh penurunan ekspor bahan bakar mineral sebesar 19,04% nilai dan 7,26% volume.
+2.  Pemerintah dan Pertamina Group mengintensifkan upaya penyaluran dan distribusi energi untuk wilayah Sumatra yang terdampak bencana banjir dan longsor di Aceh, Sumatra Utara, dan Sumatra Barat, serta dalam rangka persiapan periode Natal 2025 dan Tahun Baru 2026 (Nataru). Langkah-langkah yang diambil meliputi pengerahan armada tanker oleh PTPertamina International Shipping, penggunaan moda transportasi beragam seperti pesawat Hercules dan perintis untuk pengiriman BBM ke daerah terisolasi, serta peniadaan sementara sistem barcode MyPertamina untuk pembelian BBM subsidi di daerah bencana. Pertamina Patra Niaga juga berhasil menyuplai total 430.000 barel base fuel kepada SPBU swasta (Shell, BP-AKR, Vivo) untuk menormalisasi kembali ketersediaan BBM mereka.
+3.  Dalam pengembangan industri kilang, PT Kilang Pertamina Internasional (KPI) berkomitmen meningkatkan produksi petrokimia, dengan proyek Refinery Development Master Plan Balikpapan yang akan menghasilkan propilena sekitar 225.000 ton per tahun untuk mengurangi ketergantungan impor. Selain itu, pemerintah berencana merombak skema subsidi energi (BBM dan listrik) dalam dua tahun ke depan untuk meningkatkan efisiensi dan ketepatan sasaran. Pertamina Patra Niaga juga mempertimbangkan opsi impor Pertalite dari Amerika Serikat yang direncanakan mencapai 40% dari total pengadaan, sebagai bagian dari strategi ketahanan energi nasional.</t>
         </is>
       </c>
     </row>
@@ -2356,9 +2361,9 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.  Kementerian Energi dan Sumber Daya Mineral melaporkan Indonesia kehilangan devisa sebesar Rp523 triliun per tahun akibat impor minyak. Pada 2024, produksi minyak Indonesia mencapai 221 juta barel, sementara impor minyak nasional sebesar 313 juta barel yang mencakup 112 juta barel minyak mentah dan 201 juta barel Bahan Bakar Minyak (BBM), dengan konsumsi BBM nasional sebesar 532 juta barel. Pemerintah berupaya mengurangi ketergantungan impor melalui kebijakan seperti implementasi B50 pada 2026 dan campuran etanol 10% pada 2027, serta menolak permintaan tambahan kuota impor BBM dari SPBU swasta pada 2025 dengan mengarahkan pembelian base fuel dari PT Pertamina Patra Niaga.
-2.  Proyek Refinery Development Master Plan (RDMP) Balikpapan dijadwalkan beroperasi komersial pada 17 Desember 2025, dengan peningkatan kapasitas unit distilasi minyak mentah (CDU) dari 260.000 barel per hari (bph) menjadi 360.000 bph, yang akan meningkatkan total kapasitas CDU nasional dari 1.17 juta bph menjadi 1.26 juta bph pada akhir 2025. Sementara itu, keputusan investasi akhir (FID) untuk proyek Grass Root Refinery (GRR) Kilang Tuban yang bernilai sekitar US$20.7 miliar hingga US$24 miliar, dengan PJSC Rosneft Oil Company sebagai mitra utama, ditargetkan rampung pada akhir Desember 2025. PT Pertamina Patra Niaga juga telah menyalurkan total 430.000 barel base fuel kepada SPBU swasta per Desember 2025 untuk mengatasi kekosongan stok sebelumnya.
-3.  Distribusi BBM dan LPG di Aceh, Sumatra Utara, dan Sumatra Barat menghadapi tantangan akibat bencana alam, mendorong PT Pertamina Patra Niaga untuk mengoptimalkan berbagai moda transportasi termasuk jalur udara menggunakan pesawat Air Tractor guna memastikan pasokan energi mencapai wilayah terisolir. Kementerian Energi dan Sumber Daya Mineral memperpanjang relaksasi pembelian BBM subsidi tanpa penggunaan QR code di wilayah terdampak bencana hingga akhir Desember 2025. Selain itu, harga BBM nonsubsidi dari Pertamina, Shell, BP-AKR, dan Vivo mengalami penyesuaian kenaikan per 1 Desember 2025. Menjelang Natal dan Tahun Baru 2026, Pertamina Patra Niaga memproyeksikan kenaikan kebutuhan BBM jenis gasolin sebesar 5% dan avtur 1.6%, serta penurunan gasoil sebesar 4% di wilayah Jawa Tengah-DI Yogyakarta.</t>
+          <t>1. Kementerian Energi dan Sumber Daya Mineral (ESDM) melaporkan devisa negara hilang Rp523 triliun per tahun akibat impor minyak dan Bahan Bakar Minyak (BBM), dengan produksi minyak Indonesia 221 juta barel pada 2024 berbanding impor 313 juta barel. Sebagai upaya penahanan laju impor, Pertamina Patra Niaga telah menyalurkan 430.000 barel base fuel kepada SPBU swasta, mengakhiri kekosongan stok sejak akhir Agustus 2025. Kementerian ESDM juga akan memutuskan kuota impor BBM untuk SPBU swasta pada tahun 2026.
+2. Pertamina Patra Niaga menaikkan harga BBM nonsubsidi per 1 Desember 2025, seperti Pertamax (RON 92) menjadi Rp12.750 per liter dari sebelumnya Rp12.200 per liter, sejalan dengan tren harga minyak global dan nilai tukar rupiah terhadap dolar Amerika Serikat. SPBU swasta juga melakukan penyesuaian harga serupa. Untuk periode Natal 2025 dan Tahun Baru 2026 (Nataru), Pertamina Patra Niaga memproyeksikan kenaikan kebutuhan gasolin 5% dan avtur 1,6%, serta memberikan diskon avtur rata-rata 10% di 37 bandara strategis mulai 22 Desember 2025.
+3. Kilang Pertamina Internasional (KPI) mempercepat proyek Refinery Development Master Plan (RDMP) Balikpapan untuk meningkatkan kapasitas pengolahan minyak mentah dari 260.000 barel menjadi 360.000 barel per hari, dengan target operasi komersial pada 17 Desember 2025. Proyek ini bernilai US$7,4 miliar. Sementara itu, keputusan investasi akhir (FID) untuk proyek Grass Root Refinery (GRR) Kilang Tuban, yang bernilai US$20,7 miliar hingga US$24 miliar, diharapkan diputuskan antara Pertamina dan Rosneft Singapore Pte Ltd pada pertengahan Desember 2025.</t>
         </is>
       </c>
     </row>
@@ -2374,10 +2379,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="11.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11.90625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="10.36328125" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2422,6 +2427,163 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Tanggal awal</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Tanggal akhir</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Summary Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45950</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>45961</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>45968</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1. PT Pertamina Patra Niaga (PPN) menyalurkan 100.000 barel bahan bakar dasar impor kepada BP-AKR untuk menormalisasi pasokan BBM di SPBU swasta, dengan 100.000 barel tambahan diperkirakan tiba pada pekan ketiga November 2025. Badan usaha swasta lainnya, termasuk Vivo dan Shell, masih dalam tahap negosiasi untuk pembelian bahan bakar dasar dari Pertamina.
+2. Per 01 November 2025, Pertamina menaikkan harga Dexlite dan Pertamina Dex sebesar Rp200 per liter, menjadi Rp13.900 per liter dan Rp14.200 per liter. Pada periode yang sama, Shell dan BP-AKR juga menyesuaikan harga BBM, dengan mayoritas jenis bensin turun dan jenis diesel naik.
+3. Terkait dugaan masalah kualitas Pertalite di Jawa Timur, Pertamina Patra Niaga bersama Lemigas Kementerian ESDM melakukan pengecekan di sekitar 300 SPBU. Hasil sementara menunjukkan bahwa Pertalite yang disalurkan "on specification" tanpa kontaminasi air atau etanol, dan Pertamina telah membuka 32 posko pengaduan serta bengkel rekanan untuk memberikan solusi dan kompensasi kepada masyarakat yang terdampak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45969</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>45975</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1.  Pemerintah daerah Sumatra Barat dan Pertamina Patra Niaga telah mengambil langkah cepat untuk memulihkan kelangkaan bahan bakar minyak di wilayah tersebut pada November 2025, dengan Pertamina mempercepat pasokan melalui jalur darat dan mengoperasikan Integrated Terminal Teluk Kabung 24 jam sehari sejak 7 November 2025, yang meningkatkan kecepatan penyaluran sekitar 16%. Di sisi lain, Kementerian Energi dan Sumber Daya Mineral mendorong SPBU swasta untuk membeli base fuel dari Pertamina Patra Niaga untuk mengatasi ketimpangan pasokan, di mana BP-AKR telah sepakat membeli dua kargo atau 200.000 barel base fuel, dengan indikasi akan menambah pesanan hingga 300.000 barel, sementara Shell dan Vivo masih dalam tahap negosiasi.
+2.  Kementerian Keuangan mengawal penyelesaian Proyek Refinery Development Master Plan (RDMP) Balikpapan yang ditargetkan meningkatkan kapasitas produksi bahan bakar minyak hingga 142.000 barel per hari, LPG 336.000 ton per tahun, dan propylene 300.000 ton per tahun, dengan nilai investasi mencapai US$7,4 miliar. PT Kilang Pertamina Internasional telah melakukan pengoperasian awal Unit Residual Fluid Catalytic Cracking Complex di RDMP Balikpapan pada 10 November 2025, yang berhasil meningkatkan kapasitas pengolahan minyak mentah dari 260.000 menjadi 360.000 barel per hari dan produksi LPG menjadi 43.000 ton per tahun. Sementara itu, keputusan investasi akhir atau Final Investment Decision (FID) proyek Kilang Tuban berkapasitas 300.000 barel per hari dengan Rosneft ditargetkan rampung pada awal Desember 2025.
+3.  Kementerian Energi dan Sumber Daya Mineral mendorong penerapan bensin campuran 10% etanol (E10) pada 2028, atau berpotensi dipercepat menjadi 2027, dengan kebutuhan etanol mencapai 1,4 juta hingga 4 juta kiloliter. Proyek ini menghadapi tantangan seperti ketersediaan bahan baku, keterbatasan insentif, dan infrastruktur distribusi yang belum memadai, serta usulan dari Asosiasi Produsen Spiritus dan Etanol Indonesia untuk membebaskan etanol dari kategori barang kena cukai sebesar Rp20.000 per liter agar tidak membebani harga bensin hijau bagi konsumen. Pemerintah juga mencari keterlibatan sektor swasta, dengan Toyota Indonesia menunjukkan minat untuk mengembangkan pabrik bioetanol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>45976</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>45982</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.  Penyelesaian Proyek Refinery Development Master Plan (RDMP) Balikpapan senilai 7.4 miliar USD ditargetkan pada pertengahan Desember 2025. Proyek ini akan meningkatkan kapasitas kilang dari 260.000 barel per hari (bph) menjadi 360.000 bph, berpotensi mengurangi ketergantungan impor Bahan Bakar Minyak (BBM) hingga 15% dan memenuhi 22%-25% kebutuhan energi domestik. Unit Residual Fluid Catalytic Cracking (RFCC) Complex dengan kapasitas 90.000 bph telah mulai beroperasi pada 10 November 2025.
+2.  PT Pertamina Patra Niaga mencatat volume penjualan bensin dan solar sebesar 87 juta kiloliter (KL) per Oktober 2025, dengan 41% berasal dari produk non-subsidi. Penyaluran Solar bersubsidi terkendali 1.5% di bawah kuota 18.8 juta KL dan Pertalite 10% di bawah kuota 31.2 juta KL hingga Oktober 2025. Permintaan Pertamax Turbo (RON 98) melonjak 76%, sehingga Pertamina menambah pasokan melalui impor dan memastikan kesiapan distribusi untuk periode Natal dan Tahun Baru 2025-2026.
+3.  Dalam pengembangan biofuel, penjualan Pertamax Green 95 (E5) di 168 SPBU Pertamina mencatat pertumbuhan 80% dari 2024, dengan proyeksi kebutuhan bioetanol 4,800-5,000 KL per tahun untuk Pulau Jawa. Asosiasi Produsen Spiritus dan Etanol Indonesia (Aspendo) mengusulkan penghapusan cukai bioetanol fuel grade sebesar Rp20.000 per liter untuk menjaga harga kompetitif. Sementara itu, BP-AKR membeli 100.000 barel base fuel dari Pertamina Patra Niaga untuk mengatasi kekurangan stok, sedangkan Shell dan Vivo masih dalam negosiasi business-to-business untuk pengadaan base fuel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>45983</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>45989</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1. PT Pertamina Patra Niaga memperkuat pasokan BBM untuk periode Natal 2025 dan Tahun Baru 2026. Ini mencakup penambahan 1,4 juta kiloliter Pertalite dari produksi kilang domestik dan impor baru, dengan target ketahanan stok 21-23 hari per 25 November 2025. Kilang Pertamina Internasional juga memulai operasi awal unit Residual Fluid Catalytic Cracking (RFCC) berkapasitas 90 ribu barel per hari di Kilang Balikpapan sejak 10 November 2025, yang akan meningkatkan produksi gasoline dan LPG serta mengurangi impor.
+2. Pasokan BBM di SPBU swasta mulai normal kembali setelah mencapai kesepakatan pembelian base fuel dari Pertamina Patra Niaga. Vivo Energy Indonesia telah menerima 100.000 barel Revvo 92 (RON 92) yang mulai tersedia bertahap sejak 23 November 2025. BP-AKR menambah pembelian base fuel menjadi total 230.000 barel dari Pertamina Patra Niaga per 27 November 2025. Shell Indonesia juga menyelesaikan kesepakatan pada 25 November 2025 untuk membeli 100.000 barel base fuel, dengan harapan stok pulih akhir November 2025.
+3. Distribusi energi menghadapi tantangan cuaca ekstrem dan diperkuat dengan langkah keamanan. Dua kapal pengangkut Pertalite dan Biosolar tidak dapat bersandar di Belawan, Sumatra Utara sejak 23 November 2025 karena cuaca ekstrem, menyebabkan penyesuaian pola suplai dari terminal alternatif. Untuk mengamankan infrastruktur energi nasional, pemerintah akan mengerahkan personel TNI untuk menjaga kilang minyak dan terminal BBM Pertamina yang memiliki kapasitas pengolahan 1 juta barel per hari dan 231 terminal migas, dimulai pada Desember 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>45990</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>45991</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>45998</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1. Kilang Pertamina Internasional (KPI) menargetkan produksi untuk November 2025 sebesar 8 juta barel gasoline, 10,7 juta barel gasoil, dan 2,2 juta barel avtur. Untuk Desember 2025, produksi gasoil seri ditingkatkan menjadi sekitar 11,5 juta barel, sementara volume gasoline dan avtur dipertahankan sesuai rencana November 2025 guna mendukung kelancaran pasokan BBM menjelang periode Natal dan Tahun Baru 2026.
+2. Badan Pusat Statistik (BPS) mencatat volume ekspor bahan bakar mineral (BBM) Indonesia turun sebesar 7,26% pada Oktober 2025 dibandingkan periode yang sama tahun lalu. Penurunan ini merupakan bagian dari total ekspor migas yang turun 33,60% secara tahunan menjadi US$0,89 miliar.
+3. PT Pertamina Patra Niaga (PPN) memasok total 430.000 barel base fuel kepada badan usaha SPBU swasta seperti Shell, Vivo, dan BP-AKR untuk memastikan ketersediaan BBM. PPN juga memproyeksikan peningkatan konsumsi gasoline sebesar 8,4% dan avtur sebesar 2,4% selama periode Nataru 2025/2026 di wilayah Jawa Timur, Bali, dan Nusa Tenggara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46005</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1.  Kementerian Energi dan Sumber Daya Mineral melaporkan Indonesia kehilangan devisa sebesar Rp523 triliun per tahun akibat impor minyak. Pada 2024, produksi minyak Indonesia mencapai 221 juta barel, sementara impor minyak nasional sebesar 313 juta barel yang mencakup 112 juta barel minyak mentah dan 201 juta barel Bahan Bakar Minyak (BBM), dengan konsumsi BBM nasional sebesar 532 juta barel. Pemerintah berupaya mengurangi ketergantungan impor melalui kebijakan seperti implementasi B50 pada 2026 dan campuran etanol 10% pada 2027, serta menolak permintaan tambahan kuota impor BBM dari SPBU swasta pada 2025 dengan mengarahkan pembelian base fuel dari PT Pertamina Patra Niaga.
+2.  Proyek Refinery Development Master Plan (RDMP) Balikpapan dijadwalkan beroperasi komersial pada 17 Desember 2025, dengan peningkatan kapasitas unit distilasi minyak mentah (CDU) dari 260.000 barel per hari (bph) menjadi 360.000 bph, yang akan meningkatkan total kapasitas CDU nasional dari 1.17 juta bph menjadi 1.26 juta bph pada akhir 2025. Sementara itu, keputusan investasi akhir (FID) untuk proyek Grass Root Refinery (GRR) Kilang Tuban yang bernilai sekitar US$20.7 miliar hingga US$24 miliar, dengan PJSC Rosneft Oil Company sebagai mitra utama, ditargetkan rampung pada akhir Desember 2025. PT Pertamina Patra Niaga juga telah menyalurkan total 430.000 barel base fuel kepada SPBU swasta per Desember 2025 untuk mengatasi kekosongan stok sebelumnya.
+3.  Distribusi BBM dan LPG di Aceh, Sumatra Utara, dan Sumatra Barat menghadapi tantangan akibat bencana alam, mendorong PT Pertamina Patra Niaga untuk mengoptimalkan berbagai moda transportasi termasuk jalur udara menggunakan pesawat Air Tractor guna memastikan pasokan energi mencapai wilayah terisolir. Kementerian Energi dan Sumber Daya Mineral memperpanjang relaksasi pembelian BBM subsidi tanpa penggunaan QR code di wilayah terdampak bencana hingga akhir Desember 2025. Selain itu, harga BBM nonsubsidi dari Pertamina, Shell, BP-AKR, dan Vivo mengalami penyesuaian kenaikan per 1 Desember 2025. Menjelang Natal dan Tahun Baru 2026, Pertamina Patra Niaga memproyeksikan kenaikan kebutuhan BBM jenis gasolin sebesar 5% dan avtur 1.6%, serta penurunan gasoil sebesar 4% di wilayah Jawa Tengah-DI Yogyakarta.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2432,7 +2594,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
@@ -2486,7 +2648,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -2765,7 +2927,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -3029,7 +3191,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -3113,7 +3275,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -3197,7 +3359,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
@@ -3266,7 +3428,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">

</xml_diff>